<commit_message>
Add fabric material gallery and SKU previews
</commit_message>
<xml_diff>
--- a/data/import/fabric/fabric.xlsx
+++ b/data/import/fabric/fabric.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,16 +486,376 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>bmw-check</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>BMW Check</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW Check/FA1836.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>bmw-m-pattern</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
           <t>fabric</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>BMW M Pattern</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW M Pattern/FA5990.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>houndstooth-plaid</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Houndstooth Plaid</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Houndstooth Plaid/FA8765.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>mercedes-check</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mercedes Check </t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Check /FA8475.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>mercedes-rodeo</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Mercedes Rodeo</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Rodeo/FA8598.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>mercedes-tartan</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Mercedes Tartan</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Tartan/FA8626.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>porsche-check</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Porsche Check</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Check/FA8045.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>porsche-herringbone</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Porsche Herringbone</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Herringbone/FA3570.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>porsche-madras</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Porsche Madras</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Madras/FA8326.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>porsche-pepita</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Porsche Pepita</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8013.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>porsche-pinstripe</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Porsche Pinstripe</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3018.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>porsche-plaid</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Porsche Plaid</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Plaid/FA8525.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>porsche-script</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Porsche Script</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Script/FA3132.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>porsche-studio</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Porsche Studio </t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Studio /FA8118.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>porsche-tartan</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Porsche Tartan</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Tartan/FA8217 McLaughli.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>selected-plaid</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Selected Plaid</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Selected Plaid/FA8517.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>spirit-of-le-mans</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Spirit of Le Mans</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2002.jpg</t>
         </is>
       </c>
     </row>
@@ -648,7 +1008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -734,16 +1094,1482 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>fa1836</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>bmw-check</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>FA1836</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW Check/FA1836.jpg</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW Check/FA1836.jpg</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW Check/FA1836.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>fa5990</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
           <t>fabric</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>bmw-m-pattern</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FA5990</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW M Pattern/FA5990.jpg</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW M Pattern/FA5990.jpg</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW M Pattern/FA5990.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>fa8765</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>houndstooth-plaid</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>FA8765</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Houndstooth Plaid/FA8765.jpg</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Houndstooth Plaid/FA8765.jpg</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Houndstooth Plaid/FA8765.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>fa8475</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>mercedes-check</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>FA8475</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Check /FA8475.jpg</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Check /FA8475.jpg</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Check /FA8475.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>fa8598</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>mercedes-rodeo</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>FA8598</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Rodeo/FA8598.jpg</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Rodeo/FA8598.jpg</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Rodeo/FA8598.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>fa8626</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>mercedes-tartan</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>FA8626</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Tartan/FA8626.jpg</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Tartan/FA8626.jpg</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Tartan/FA8626.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>fa8637</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>mercedes-tartan</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>FA8637</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Tartan/FA8637.jpg</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Tartan/FA8637.jpg</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Tartan/FA8637.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>fa8045</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>porsche-check</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>FA8045</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Check/FA8045.jpg</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Check/FA8045.jpg</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Check/FA8045.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>fa8057</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>porsche-check</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>FA8057</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Check/FA8057.jpg</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Check/FA8057.jpg</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Check/FA8057.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>fa8063</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>porsche-check</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>FA8063</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Check/FA8063.jpg</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Check/FA8063.jpg</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Check/FA8063.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>fa3570</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>porsche-herringbone</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>FA3570</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Herringbone/FA3570.jpg</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Herringbone/FA3570.jpg</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Herringbone/FA3570.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>fa8326</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>porsche-madras</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>FA8326</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Madras/FA8326.jpg</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Madras/FA8326.jpg</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Madras/FA8326.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>fa8354</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>porsche-madras</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>FA8354</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Madras/FA8354.jpg</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Madras/FA8354.jpg</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Madras/FA8354.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>fa8013</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>porsche-pepita</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>FA8013</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8013.jpg</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8013.jpg</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8013.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>fa8026</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>porsche-pepita</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>FA8026</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8026.jpg</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8026.jpg</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8026.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>fa8065</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>porsche-pepita</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>FA8065</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8065.jpg</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8065.jpg</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8065.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>fa8074</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>porsche-pepita</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>FA8074</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8074.jpg</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8074.jpg</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8074.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>fa8093</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>porsche-pepita</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>FA8093</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8093.jpg</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8093.jpg</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8093.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>fa8094</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>porsche-pepita</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>FA8094</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8094.jpg</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8094.jpg</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8094.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>fa3018</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>porsche-pinstripe</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>FA3018</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3018.jpg</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3018.jpg</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3018.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>fa3055</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>porsche-pinstripe</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>FA3055</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3055.jpg</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3055.jpg</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3055.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>fa3067</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>porsche-pinstripe</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>FA3067</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3067.jpg</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3067.jpg</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3067.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>fa3074</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>porsche-pinstripe</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>FA3074</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3074.jpg</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3074.jpg</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3074.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>fa8525</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>porsche-plaid</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>FA8525</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Plaid/FA8525.jpg</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Plaid/FA8525.jpg</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Plaid/FA8525.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>fa3132</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>porsche-script</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>FA3132</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Script/FA3132.jpg</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Script/FA3132.jpg</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Script/FA3132.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>fa3217</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>porsche-script</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>FA3217</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Script/FA3217.jpg</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Script/FA3217.jpg</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Script/FA3217.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>fa3258</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>porsche-script</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>FA3258</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Script/FA3258.jpg</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Script/FA3258.jpg</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Script/FA3258.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>fa3272</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>porsche-script</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>FA3272</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Script/FA3272.jpg</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Script/FA3272.jpg</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Script/FA3272.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>fa8118</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>porsche-studio</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>FA8118</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Studio /FA8118.jpg</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Studio /FA8118.jpg</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Studio /FA8118.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fa8128</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>porsche-studio</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>FA8128</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Studio /FA8128.jpg</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Studio /FA8128.jpg</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Studio /FA8128.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>fa8165</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>porsche-studio</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>FA8165</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Studio /FA8165.jpg</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Studio /FA8165.jpg</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Studio /FA8165.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>fa8166</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>porsche-studio</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>FA8166</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Studio /FA8166.jpg</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Studio /FA8166.jpg</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Studio /FA8166.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>fa8217</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>porsche-tartan</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>FA8217</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Tartan/FA8217 McLaughli.jpg</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Tartan/FA8217 McLaughli.jpg</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Tartan/FA8217 McLaughli.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>fa8237</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>porsche-tartan</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>FA8237</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Tartan/FA8237 Black Watch.jpg</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Tartan/FA8237 Black Watch.jpg</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Tartan/FA8237 Black Watch.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>fa8271</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>porsche-tartan</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>FA8271</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Tartan/FA8271 Mackenzie.jpg</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Tartan/FA8271 Mackenzie.jpg</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Tartan/FA8271 Mackenzie.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>fa8517</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>selected-plaid</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>FA8517</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Selected Plaid/FA8517.jpg</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Selected Plaid/FA8517.jpg</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Selected Plaid/FA8517.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>fa8553</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>selected-plaid</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>FA8553</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Selected Plaid/FA8553.jpg</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Selected Plaid/FA8553.jpg</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Selected Plaid/FA8553.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>fa2002</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>spirit-of-le-mans</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>FA2002</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2002.jpg</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2002.jpg</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2002.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>fa2202</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>spirit-of-le-mans</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>FA2202</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2202.jpg</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2202.jpg</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2202.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>fa2729</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>spirit-of-le-mans</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>FA2729</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2729.jpg</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2729.jpg</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2729.jpg</t>
         </is>
       </c>
     </row>
@@ -860,7 +2686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -890,6 +2716,606 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>fa1836</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW Check/FA1836.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>fa5990</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW M Pattern/FA5990.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>fa8765</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Houndstooth Plaid/FA8765.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>fa8475</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Check /FA8475.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>fa8598</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Rodeo/FA8598.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>fa8626</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Tartan/FA8626.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>fa8637</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Tartan/FA8637.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>fa8045</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Check/FA8045.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>fa8057</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Check/FA8057.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>fa8063</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Check/FA8063.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>fa3570</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Herringbone/FA3570.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>fa8326</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Madras/FA8326.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>fa8354</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Madras/FA8354.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>fa8013</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8013.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>fa8026</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8026.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>fa8065</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8065.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>fa8074</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8074.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>fa8093</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8093.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>fa8094</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pepita/FA8094.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>fa3018</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3018.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>fa3055</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3055.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>fa3067</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3067.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>fa3074</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3074.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>fa8525</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Plaid/FA8525.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>fa3132</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Script/FA3132.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>fa3217</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Script/FA3217.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>fa3258</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Script/FA3258.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>fa3272</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Script/FA3272.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>fa8118</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Studio /FA8118.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fa8128</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Studio /FA8128.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>fa8165</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Studio /FA8165.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>fa8166</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Studio /FA8166.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>fa8217</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Tartan/FA8217 McLaughli.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>fa8237</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Tartan/FA8237 Black Watch.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>fa8271</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Porsche Tartan/FA8271 Mackenzie.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>fa8517</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Selected Plaid/FA8517.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>fa8553</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Selected Plaid/FA8553.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>fa2002</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2002.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>fa2202</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2202.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>fa2729</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2729.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add fabric cover and hover preview images
</commit_message>
<xml_diff>
--- a/data/import/fabric/fabric.xlsx
+++ b/data/import/fabric/fabric.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>/uploads/fabric/BMW Check/FA1836.jpg</t>
+          <t>/uploads/fabric/Cover/FA1836.jpg</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>/uploads/fabric/BMW M Pattern/FA5990.jpg</t>
+          <t>/uploads/fabric/Cover/FA5990.jpg</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Houndstooth Plaid/FA8765.jpg</t>
+          <t>/uploads/fabric/Cover/FA8765.jpg</t>
         </is>
       </c>
     </row>
@@ -569,7 +569,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Mercedes Check /FA8475.jpg</t>
+          <t>/uploads/fabric/Cover/FA8475.jpg</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Mercedes Rodeo/FA8598.jpg</t>
+          <t>/uploads/fabric/Cover/FA8598.jpg</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Mercedes Tartan/FA8626.jpg</t>
+          <t>/uploads/fabric/Cover/FA8626.jpg</t>
         </is>
       </c>
     </row>
@@ -635,7 +635,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Check/FA8045.jpg</t>
+          <t>/uploads/fabric/Cover/FA8045.jpg</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Herringbone/FA3570.jpg</t>
+          <t>/uploads/fabric/Cover/FA3570.jpg</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Madras/FA8326.jpg</t>
+          <t>/uploads/fabric/Cover/FA8326.jpg</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Pepita/FA8013.jpg</t>
+          <t>/uploads/fabric/Cover/FA8013.jpg</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Pinstripe/FA3018.jpg</t>
+          <t>/uploads/fabric/Cover/FA3018.jpg</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Plaid/FA8525.jpg</t>
+          <t>/uploads/fabric/Cover/FA8525.jpg</t>
         </is>
       </c>
     </row>
@@ -767,7 +767,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Script/FA3132.jpg</t>
+          <t>/uploads/fabric/Cover/FA3132.jpg</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Studio /FA8118.jpg</t>
+          <t>/uploads/fabric/Cover/FA8118.jpg</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Tartan/FA8217 McLaughli.jpg</t>
+          <t>/uploads/fabric/Cover/FA8217.jpg</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Selected Plaid/FA8517.jpg</t>
+          <t>/uploads/fabric/Cover/FA8517.jpg</t>
         </is>
       </c>
     </row>
@@ -855,7 +855,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Spirit of Le Mans/FA2002.jpg</t>
+          <t>/uploads/fabric/Cover/FA2002.jpg</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P41"/>
+  <dimension ref="A1:Q41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1059,35 +1059,40 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>preview_image</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>summary_en</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>summary_ja</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>seo_title_en</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>seo_title_ja</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>seo_description_en</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>seo_description_ja</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>seo_image</t>
         </is>
@@ -1124,7 +1129,12 @@
           <t>/uploads/fabric/BMW Check/FA1836.jpg</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA1836.jpg</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>/uploads/fabric/BMW Check/FA1836.jpg</t>
         </is>
@@ -1161,7 +1171,12 @@
           <t>/uploads/fabric/BMW M Pattern/FA5990.jpg</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA5990.jpg</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>/uploads/fabric/BMW M Pattern/FA5990.jpg</t>
         </is>
@@ -1198,7 +1213,12 @@
           <t>/uploads/fabric/Houndstooth Plaid/FA8765.jpg</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8765.jpg</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>/uploads/fabric/Houndstooth Plaid/FA8765.jpg</t>
         </is>
@@ -1235,7 +1255,12 @@
           <t>/uploads/fabric/Mercedes Check /FA8475.jpg</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8475.jpg</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>/uploads/fabric/Mercedes Check /FA8475.jpg</t>
         </is>
@@ -1272,7 +1297,12 @@
           <t>/uploads/fabric/Mercedes Rodeo/FA8598.jpg</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8598.jpg</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>/uploads/fabric/Mercedes Rodeo/FA8598.jpg</t>
         </is>
@@ -1309,7 +1339,12 @@
           <t>/uploads/fabric/Mercedes Tartan/FA8626.jpg</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8626.jpg</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>/uploads/fabric/Mercedes Tartan/FA8626.jpg</t>
         </is>
@@ -1346,7 +1381,12 @@
           <t>/uploads/fabric/Mercedes Tartan/FA8637.jpg</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8637.jpg</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>/uploads/fabric/Mercedes Tartan/FA8637.jpg</t>
         </is>
@@ -1383,7 +1423,12 @@
           <t>/uploads/fabric/Porsche Check/FA8045.jpg</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8045.jpg</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Check/FA8045.jpg</t>
         </is>
@@ -1420,7 +1465,12 @@
           <t>/uploads/fabric/Porsche Check/FA8057.jpg</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8057.jpg</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Check/FA8057.jpg</t>
         </is>
@@ -1457,7 +1507,12 @@
           <t>/uploads/fabric/Porsche Check/FA8063.jpg</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8063.jpg</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Check/FA8063.jpg</t>
         </is>
@@ -1494,7 +1549,12 @@
           <t>/uploads/fabric/Porsche Herringbone/FA3570.jpg</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA3570.jpg</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Herringbone/FA3570.jpg</t>
         </is>
@@ -1531,7 +1591,12 @@
           <t>/uploads/fabric/Porsche Madras/FA8326.jpg</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8326.jpg</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Madras/FA8326.jpg</t>
         </is>
@@ -1568,7 +1633,12 @@
           <t>/uploads/fabric/Porsche Madras/FA8354.jpg</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8354.jpg</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Madras/FA8354.jpg</t>
         </is>
@@ -1605,7 +1675,12 @@
           <t>/uploads/fabric/Porsche Pepita/FA8013.jpg</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8013.jpg</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pepita/FA8013.jpg</t>
         </is>
@@ -1642,7 +1717,12 @@
           <t>/uploads/fabric/Porsche Pepita/FA8026.jpg</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8026.jpg</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pepita/FA8026.jpg</t>
         </is>
@@ -1679,7 +1759,12 @@
           <t>/uploads/fabric/Porsche Pepita/FA8065.jpg</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8065.jpg</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pepita/FA8065.jpg</t>
         </is>
@@ -1716,7 +1801,12 @@
           <t>/uploads/fabric/Porsche Pepita/FA8074.jpg</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8074.jpg</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pepita/FA8074.jpg</t>
         </is>
@@ -1753,7 +1843,12 @@
           <t>/uploads/fabric/Porsche Pepita/FA8093.jpg</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8093.jpg</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pepita/FA8093.jpg</t>
         </is>
@@ -1790,7 +1885,12 @@
           <t>/uploads/fabric/Porsche Pepita/FA8094.jpg</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8094.jpg</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pepita/FA8094.jpg</t>
         </is>
@@ -1827,7 +1927,12 @@
           <t>/uploads/fabric/Porsche Pinstripe/FA3018.jpg</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA3018.jpg</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pinstripe/FA3018.jpg</t>
         </is>
@@ -1864,7 +1969,12 @@
           <t>/uploads/fabric/Porsche Pinstripe/FA3055.jpg</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA3055.jpg</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pinstripe/FA3055.jpg</t>
         </is>
@@ -1901,7 +2011,12 @@
           <t>/uploads/fabric/Porsche Pinstripe/FA3067.jpg</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA3067.jpg</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pinstripe/FA3067.jpg</t>
         </is>
@@ -1938,7 +2053,12 @@
           <t>/uploads/fabric/Porsche Pinstripe/FA3074.jpg</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA3074.jpg</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pinstripe/FA3074.jpg</t>
         </is>
@@ -1975,7 +2095,12 @@
           <t>/uploads/fabric/Porsche Plaid/FA8525.jpg</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8525.jpg</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Plaid/FA8525.jpg</t>
         </is>
@@ -2012,7 +2137,12 @@
           <t>/uploads/fabric/Porsche Script/FA3132.jpg</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA3132.jpg</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Script/FA3132.jpg</t>
         </is>
@@ -2049,7 +2179,12 @@
           <t>/uploads/fabric/Porsche Script/FA3217.jpg</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA3217.jpg</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Script/FA3217.jpg</t>
         </is>
@@ -2086,7 +2221,12 @@
           <t>/uploads/fabric/Porsche Script/FA3258.jpg</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA3258.jpg</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Script/FA3258.jpg</t>
         </is>
@@ -2123,7 +2263,12 @@
           <t>/uploads/fabric/Porsche Script/FA3272.jpg</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA3272.jpg</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Script/FA3272.jpg</t>
         </is>
@@ -2160,7 +2305,12 @@
           <t>/uploads/fabric/Porsche Studio /FA8118.jpg</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8118.jpg</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Studio /FA8118.jpg</t>
         </is>
@@ -2197,7 +2347,12 @@
           <t>/uploads/fabric/Porsche Studio /FA8128.jpg</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr">
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8128.jpg</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Studio /FA8128.jpg</t>
         </is>
@@ -2234,7 +2389,12 @@
           <t>/uploads/fabric/Porsche Studio /FA8165.jpg</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8165.jpg</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Studio /FA8165.jpg</t>
         </is>
@@ -2271,7 +2431,8 @@
           <t>/uploads/fabric/Porsche Studio /FA8166.jpg</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr">
+      <c r="J33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Studio /FA8166.jpg</t>
         </is>
@@ -2308,7 +2469,12 @@
           <t>/uploads/fabric/Porsche Tartan/FA8217 McLaughli.jpg</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr">
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8217.jpg</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Tartan/FA8217 McLaughli.jpg</t>
         </is>
@@ -2345,7 +2511,12 @@
           <t>/uploads/fabric/Porsche Tartan/FA8237 Black Watch.jpg</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr">
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8237.jpg</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Tartan/FA8237 Black Watch.jpg</t>
         </is>
@@ -2382,7 +2553,12 @@
           <t>/uploads/fabric/Porsche Tartan/FA8271 Mackenzie.jpg</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr">
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8271.jpg</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Tartan/FA8271 Mackenzie.jpg</t>
         </is>
@@ -2419,7 +2595,12 @@
           <t>/uploads/fabric/Selected Plaid/FA8517.jpg</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr">
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8517.jpg</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
         <is>
           <t>/uploads/fabric/Selected Plaid/FA8517.jpg</t>
         </is>
@@ -2456,7 +2637,12 @@
           <t>/uploads/fabric/Selected Plaid/FA8553.jpg</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr">
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8553.jpg</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
         <is>
           <t>/uploads/fabric/Selected Plaid/FA8553.jpg</t>
         </is>
@@ -2493,7 +2679,12 @@
           <t>/uploads/fabric/Spirit of Le Mans/FA2002.jpg</t>
         </is>
       </c>
-      <c r="P39" t="inlineStr">
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA2002.jpg</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
         <is>
           <t>/uploads/fabric/Spirit of Le Mans/FA2002.jpg</t>
         </is>
@@ -2530,7 +2721,12 @@
           <t>/uploads/fabric/Spirit of Le Mans/FA2202.jpg</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr">
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA2202.jpg</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
         <is>
           <t>/uploads/fabric/Spirit of Le Mans/FA2202.jpg</t>
         </is>
@@ -2567,7 +2763,12 @@
           <t>/uploads/fabric/Spirit of Le Mans/FA2729.jpg</t>
         </is>
       </c>
-      <c r="P41" t="inlineStr">
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA2729.jpg</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
         <is>
           <t>/uploads/fabric/Spirit of Le Mans/FA2729.jpg</t>
         </is>

</xml_diff>

<commit_message>
Add missing FA8166 fabric preview assets
</commit_message>
<xml_diff>
--- a/data/import/fabric/fabric.xlsx
+++ b/data/import/fabric/fabric.xlsx
@@ -2431,7 +2431,11 @@
           <t>/uploads/fabric/Porsche Studio /FA8166.jpg</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8166.jpg</t>
+        </is>
+      </c>
       <c r="Q33" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Studio /FA8166.jpg</t>

</xml_diff>

<commit_message>
Add fabric case gallery images
</commit_message>
<xml_diff>
--- a/data/import/fabric/fabric.xlsx
+++ b/data/import/fabric/fabric.xlsx
@@ -2932,7 +2932,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>/uploads/fabric/BMW Check/FA1836.jpg</t>
+          <t>/uploads/fabric/Case/FA1836.jpg</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>/uploads/fabric/BMW M Pattern/FA5990.jpg</t>
+          <t>/uploads/fabric/Case/FA5990.jpg</t>
         </is>
       </c>
     </row>
@@ -2962,7 +2962,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Houndstooth Plaid/FA8765.jpg</t>
+          <t>/uploads/fabric/Case/FA8765.jpg</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Mercedes Check /FA8475.jpg</t>
+          <t>/uploads/fabric/Case/FA8475.jpg</t>
         </is>
       </c>
     </row>
@@ -2992,7 +2992,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Mercedes Rodeo/FA8598.jpg</t>
+          <t>/uploads/fabric/Case/FA8598.jpg</t>
         </is>
       </c>
     </row>
@@ -3007,7 +3007,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Mercedes Tartan/FA8626.jpg</t>
+          <t>/uploads/fabric/Case/FA8626.jpg</t>
         </is>
       </c>
     </row>
@@ -3022,7 +3022,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Mercedes Tartan/FA8637.jpg</t>
+          <t>/uploads/fabric/Case/FA8637.jpg</t>
         </is>
       </c>
     </row>
@@ -3037,7 +3037,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Check/FA8045.jpg</t>
+          <t>/uploads/fabric/Case/FA8045.jpg</t>
         </is>
       </c>
     </row>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Check/FA8057.jpg</t>
+          <t>/uploads/fabric/Case/FA8057.jpg</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3067,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Check/FA8063.jpg</t>
+          <t>/uploads/fabric/Case/FA8063.jpg</t>
         </is>
       </c>
     </row>
@@ -3082,7 +3082,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Herringbone/FA3570.jpg</t>
+          <t>/uploads/fabric/Case/FA3570.jpg</t>
         </is>
       </c>
     </row>
@@ -3097,7 +3097,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Madras/FA8326.jpg</t>
+          <t>/uploads/fabric/Case/FA8326.jpg</t>
         </is>
       </c>
     </row>
@@ -3112,7 +3112,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Madras/FA8354.jpg</t>
+          <t>/uploads/fabric/Case/FA8354.jpg</t>
         </is>
       </c>
     </row>
@@ -3127,7 +3127,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Pepita/FA8013.jpg</t>
+          <t>/uploads/fabric/Case/FA8013.jpg</t>
         </is>
       </c>
     </row>
@@ -3142,7 +3142,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Pepita/FA8026.jpg</t>
+          <t>/uploads/fabric/Case/FA8026.jpg</t>
         </is>
       </c>
     </row>
@@ -3157,7 +3157,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Pepita/FA8065.jpg</t>
+          <t>/uploads/fabric/Case/FA8065.jpg</t>
         </is>
       </c>
     </row>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Pepita/FA8074.jpg</t>
+          <t>/uploads/fabric/Case/FA8074.jpg</t>
         </is>
       </c>
     </row>
@@ -3187,7 +3187,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Pepita/FA8093.jpg</t>
+          <t>/uploads/fabric/Case/FA8093.jpg</t>
         </is>
       </c>
     </row>
@@ -3202,7 +3202,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Pepita/FA8094.jpg</t>
+          <t>/uploads/fabric/Case/FA8094.jpg</t>
         </is>
       </c>
     </row>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Pinstripe/FA3018.jpg</t>
+          <t>/uploads/fabric/Case/FA3018.jpg</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3232,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Pinstripe/FA3055.jpg</t>
+          <t>/uploads/fabric/Case/FA3055.jpg</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Pinstripe/FA3067.jpg</t>
+          <t>/uploads/fabric/Case/FA3067.jpg</t>
         </is>
       </c>
     </row>
@@ -3262,7 +3262,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Pinstripe/FA3074.jpg</t>
+          <t>/uploads/fabric/Case/FA3074.jpg</t>
         </is>
       </c>
     </row>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Plaid/FA8525.jpg</t>
+          <t>/uploads/fabric/Case/FA8525.jpg</t>
         </is>
       </c>
     </row>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Script/FA3132.jpg</t>
+          <t>/uploads/fabric/Case/FA3132.jpg</t>
         </is>
       </c>
     </row>
@@ -3307,7 +3307,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Script/FA3217.jpg</t>
+          <t>/uploads/fabric/Case/FA3217.jpg</t>
         </is>
       </c>
     </row>
@@ -3322,7 +3322,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Script/FA3258.jpg</t>
+          <t>/uploads/fabric/Case/FA3258.jpg</t>
         </is>
       </c>
     </row>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Script/FA3272.jpg</t>
+          <t>/uploads/fabric/Case/FA3272.jpg</t>
         </is>
       </c>
     </row>
@@ -3352,7 +3352,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Studio /FA8118.jpg</t>
+          <t>/uploads/fabric/Case/FA8118.jpg</t>
         </is>
       </c>
     </row>
@@ -3367,7 +3367,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Studio /FA8128.jpg</t>
+          <t>/uploads/fabric/Case/FA8128.jpg</t>
         </is>
       </c>
     </row>
@@ -3382,7 +3382,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Studio /FA8165.jpg</t>
+          <t>/uploads/fabric/Case/FA8165.jpg</t>
         </is>
       </c>
     </row>
@@ -3397,7 +3397,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Studio /FA8166.jpg</t>
+          <t>/uploads/fabric/Case/FA8166.jpg</t>
         </is>
       </c>
     </row>
@@ -3412,7 +3412,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Tartan/FA8217 McLaughli.jpg</t>
+          <t>/uploads/fabric/Case/FA8217.jpg</t>
         </is>
       </c>
     </row>
@@ -3427,7 +3427,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Tartan/FA8237 Black Watch.jpg</t>
+          <t>/uploads/fabric/Case/FA8237.jpg</t>
         </is>
       </c>
     </row>
@@ -3442,7 +3442,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Tartan/FA8271 Mackenzie.jpg</t>
+          <t>/uploads/fabric/Case/FA8271.jpg</t>
         </is>
       </c>
     </row>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Selected Plaid/FA8517.jpg</t>
+          <t>/uploads/fabric/Case/FA8517.jpg</t>
         </is>
       </c>
     </row>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Selected Plaid/FA8553.jpg</t>
+          <t>/uploads/fabric/Case/FA8553.jpg</t>
         </is>
       </c>
     </row>
@@ -3487,7 +3487,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Spirit of Le Mans/FA2002.jpg</t>
+          <t>/uploads/fabric/Case/FA2002.jpg</t>
         </is>
       </c>
     </row>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Spirit of Le Mans/FA2202.jpg</t>
+          <t>/uploads/fabric/Case/FA2202.jpg</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3517,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Spirit of Le Mans/FA2729.jpg</t>
+          <t>/uploads/fabric/Case/FA2729.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync fabric SEO data to Sanity
</commit_message>
<xml_diff>
--- a/data/import/fabric/fabric.xlsx
+++ b/data/import/fabric/fabric.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="320" yWindow="780" windowWidth="33900" windowHeight="19660" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="product_types" sheetId="1" state="visible" r:id="rId1"/>
@@ -17,18 +16,48 @@
     <sheet name="sku_case_gallery" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="5">
     <font>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
       <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="SimSun"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <sz val="9"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
@@ -53,11 +82,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -420,8 +461,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:O22"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <cols>
+    <col width="37" customWidth="1" min="1" max="1"/>
+    <col width="24.33203125" customWidth="1" min="3" max="3"/>
+    <col width="17.83203125" customWidth="1" min="4" max="4"/>
+    <col width="47.33203125" customWidth="1" min="5" max="5"/>
+    <col width="18.6640625" customWidth="1" min="6" max="6"/>
+    <col width="33.5" customWidth="1" min="7" max="7"/>
+    <col width="17.33203125" customWidth="1" min="8" max="8"/>
+    <col width="38.5" customWidth="1" min="9" max="9"/>
+    <col width="21.83203125" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -485,379 +537,838 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="135" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>bmw-check</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>BMW Check</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>BMW CHECK</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Classic Scottish square pattern for BMW Isetta</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>BMW Isetta Classic Tartan Seat Upholstery Fabric</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>Authentic flatwoven green Scottish square fabric for BMW Isetta restoration (models up to 1958).Exact OEM match pattern. Inquire for rolls.</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA1836.jpg</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="1" t="n"/>
+      <c r="O2" s="1" t="n"/>
+    </row>
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>bmw-m-pattern</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>BMW M Pattern</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>BMW M PATTERN</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>The M-Stripe seat cloth is a  replica of the original material used in the prototype M8.</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>BMW Seat Fabric with Foam</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>Premium reproduction of the iconic M Jahre M-Stripe seat fabric. A replica of the ultra-rare material found in the legendary M8 Prototype cabin.</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA5990.jpg</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="L3" s="1" t="n"/>
+      <c r="M3" s="1" t="n"/>
+      <c r="N3" s="1" t="n"/>
+      <c r="O3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="165" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>houndstooth-plaid</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Houndstooth Plaid</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>HOUNDSTOOTH PLAID</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="n"/>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>This textile features an intricate houndstooth-based Glen plaid layout blended with Scottish Squares for seat upholstery</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="n"/>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Houndstooth based Glen plaid with Tartan for Seat Upholstery</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="n"/>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t>Premium automotive seat upholstery featuring an intricate houndstooth-based Glen plaid layout blended with Scottish squares. Perfect for vintage car restoration.</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="n"/>
+      <c r="K4" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8765.jpg</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="L4" s="1" t="n"/>
+      <c r="M4" s="1" t="n"/>
+      <c r="N4" s="1" t="n"/>
+      <c r="O4" s="1" t="n"/>
+    </row>
+    <row r="5" ht="75" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>mercedes-check</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mercedes Check </t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MERCEDES CHECK </t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="n"/>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>This premium, original-specification automotive interior textile is an authentic factory-match reproduction of the classic first-generation Mercedes-Benz W460 G-Klasse (G-Wagon)</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="n"/>
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t>Vintage Mercedes G-Wagon Seat Upholstery Fabric</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="n"/>
+      <c r="I5" s="1" t="inlineStr">
+        <is>
+          <t>Authentic 1980s Mercedes W460 G-class seat upholstery fabric. Heavy-duty flatwoven Panamabond square design in Beige Black</t>
+        </is>
+      </c>
+      <c r="J5" s="1" t="n"/>
+      <c r="K5" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8475.jpg</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="L5" s="1" t="n"/>
+      <c r="M5" s="1" t="n"/>
+      <c r="N5" s="1" t="n"/>
+      <c r="O5" s="1" t="n"/>
+    </row>
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>mercedes-rodeo</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Mercedes Rodeo</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>MERCEDES RODEO</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="n"/>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>This premium, original-specification automotive interior textile is an authentic factory-match reproduction of the late 1980's Mercedes-Benz G-Klasse. The same pattern is used in 2025 G550 'Stronger Than the 1980s" Special Edition</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="n"/>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>Mercedes G-Wagon 'Stronger Than the 1980s'  Seat Fabric</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="n"/>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>Get the look of the limited edition G550 Stronger Than the 1980s cabin. Authentic Mercedes Rodeo Grey-Black cube upholstery fabric</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="n"/>
+      <c r="K6" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8598.jpg</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="L6" s="1" t="n"/>
+      <c r="M6" s="1" t="n"/>
+      <c r="N6" s="1" t="n"/>
+      <c r="O6" s="1" t="n"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>mercedes-tartan</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Mercedes Tartan</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>MERCEDES TARTAN</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="n"/>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Woven from 100% pure wool, this elite fabric is engineered exclusively for interior restoration of the legendary Mercedes-Benz W198 300SL Gullwing</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="n"/>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>Mercedes W198 300SL Gullwing 100% Wool Fabric</t>
+        </is>
+      </c>
+      <c r="H7" s="1" t="n"/>
+      <c r="I7" s="1" t="inlineStr">
+        <is>
+          <t>Authentic 100% wool 1954-1963 Mercedes-Benz W198 300SL Gullwing seat fabric. Factory-match blue/grey Scottish square tartan</t>
+        </is>
+      </c>
+      <c r="J7" s="1" t="n"/>
+      <c r="K7" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8626.jpg</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="L7" s="1" t="n"/>
+      <c r="M7" s="1" t="n"/>
+      <c r="N7" s="1" t="n"/>
+      <c r="O7" s="1" t="n"/>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>porsche-check</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Porsche Check</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>PORSCHE CHECK</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="n"/>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Classic pattern Porsche upholstery fabric</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="n"/>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vintage Porsche Seating Upholstery Fabric </t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="n"/>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vintage Porsche Seating Upholstery Fabric </t>
+        </is>
+      </c>
+      <c r="J8" s="1" t="n"/>
+      <c r="K8" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8045.jpg</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="L8" s="1" t="n"/>
+      <c r="M8" s="1" t="n"/>
+      <c r="N8" s="1" t="n"/>
+      <c r="O8" s="1" t="n"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>porsche-herringbone</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Porsche Herringbone</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>PORSCHE HERRINGBONE</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="n"/>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>This authentic, OEM-specification automotive seating textile is an exact factory-match reproduction for the upholstery of Porsche 924</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="n"/>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vintage Porsche Seating Upholstery Fabric Herringbone </t>
+        </is>
+      </c>
+      <c r="H9" s="1" t="n"/>
+      <c r="I9" s="1" t="inlineStr">
+        <is>
+          <t>Authentic 1978 Porsche 924 seat upholstery fabric. Premium factory-match Beige Cream Black herringbone textile</t>
+        </is>
+      </c>
+      <c r="J9" s="1" t="n"/>
+      <c r="K9" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA3570.jpg</t>
         </is>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="L9" s="1" t="n"/>
+      <c r="M9" s="1" t="n"/>
+      <c r="N9" s="1" t="n"/>
+      <c r="O9" s="1" t="n"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>porsche-madras</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Porsche Madras</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>PORSCHE MADRAS</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="n"/>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>This is the heritage seat upholstery fabric originally offered by Stuttgart as an exclusive cabin option between 1972 and 1975 used in early G-Model Porsche 911s (including the 911T, E, S, and early Carrera).</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="n"/>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>Porsche 911 Madras Seat Upholstery Fabric</t>
+        </is>
+      </c>
+      <c r="H10" s="1" t="n"/>
+      <c r="I10" s="1" t="inlineStr">
+        <is>
+          <t>Authentic 1972-1975 Porsche 911 Madras seat fabric. Premium factory-match windowpane plaid for vintage F-Model &amp; G-Model Carrera restorations</t>
+        </is>
+      </c>
+      <c r="J10" s="1" t="n"/>
+      <c r="K10" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8326.jpg</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="L10" s="1" t="n"/>
+      <c r="M10" s="1" t="n"/>
+      <c r="N10" s="1" t="n"/>
+      <c r="O10" s="1" t="n"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>porsche-pepita</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Porsche Pepita</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>PORSCHE PEPITA</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="n"/>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>Porsche Pepita is arguably the most famous, style-defining interior textile in sports car history. Officially introduced in 1965 for the original 911, Pepita originated as a special-request option for late-model Porsche 356 classics in the early 1960s.</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="n"/>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>Porsche Classic Pepita Fabric | Heritage Design Seat Upholstery</t>
+        </is>
+      </c>
+      <c r="H11" s="1" t="n"/>
+      <c r="I11" s="1" t="inlineStr">
+        <is>
+          <t>Authentic black &amp; white Porsche Pepita seat fabric. Premium factory-match pattern for classic 911 restorations and modern Heritage Design upgrades. More colors available.</t>
+        </is>
+      </c>
+      <c r="J11" s="1" t="n"/>
+      <c r="K11" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8013.jpg</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="L11" s="1" t="n"/>
+      <c r="M11" s="1" t="n"/>
+      <c r="N11" s="1" t="n"/>
+      <c r="O11" s="1" t="n"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>porsche-pinstripe</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Porsche Pinstripe</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>PORSCHE PINSTRIPE</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="n"/>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Porsche Pinstripe is a highly sophisticated, business-suit-inspired executive textile that defined the interiors of late-1970s and 1980s Porsche sports cars. It became a staple option across the air-cooled 911 (G-Model) series and the entire front-engine transaxle family (924, 944, and 928)</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="n"/>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>Vintage Porsche Pinstripe Seat Upholstery Fabric</t>
+        </is>
+      </c>
+      <c r="H12" s="1" t="n"/>
+      <c r="I12" s="1" t="inlineStr">
+        <is>
+          <t>Authentic 1977-1990 Porsche Pinstripe seat fabric. Premium factory-match flannel for classic 911, 924, 928, and 944 cabin restoration.</t>
+        </is>
+      </c>
+      <c r="J12" s="1" t="n"/>
+      <c r="K12" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA3018.jpg</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="L12" s="1" t="n"/>
+      <c r="M12" s="1" t="n"/>
+      <c r="N12" s="1" t="n"/>
+      <c r="O12" s="1" t="n"/>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>porsche-plaid</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Porsche Plaid</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>PORSCHE PLAID</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="n"/>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>This is a premium 100% wool flatwoven plaid fabric replicated for the 1973 Porsche 911 RSR</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="n"/>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t>Vintage Porsche Blue Plaid Fabric - 100% Wool Flatwoven Twill</t>
+        </is>
+      </c>
+      <c r="H13" s="1" t="n"/>
+      <c r="I13" s="1" t="inlineStr">
+        <is>
+          <t>Discover premium 100% wool automotive fabric featuring the classic 1970s Porsche RSR blue tartan pattern. Durable, period-correct woven cloth for luxury interiors.</t>
+        </is>
+      </c>
+      <c r="J13" s="1" t="n"/>
+      <c r="K13" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8525.jpg</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>porsche-script</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
+      <c r="L13" s="1" t="n"/>
+      <c r="M13" s="1" t="n"/>
+      <c r="N13" s="1" t="n"/>
+      <c r="O13" s="1" t="n"/>
+    </row>
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>porsche-velours-pinstripe</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Porsche Script</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>PORSCHE VELOURS PINSTRIPE</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="n"/>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>It is a velvet-like fabric featuring a dense, cut-pile surface. This gives it an incredibly plush, soft-touch texture that was highly favored for luxury and executive sports car cabins in the 1980s</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="n"/>
+      <c r="G14" s="1" t="inlineStr">
+        <is>
+          <t>Porsche 911 928 944 Pinstripe Velour Seat Cloth</t>
+        </is>
+      </c>
+      <c r="H14" s="1" t="n"/>
+      <c r="I14" s="1" t="inlineStr">
+        <is>
+          <t>Vintage-style vertical pinstripe velour fabric for classic Porsche interiors. Perfect for high-end seat insert and door card restorations.</t>
+        </is>
+      </c>
+      <c r="J14" s="1" t="n"/>
+      <c r="K14" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA3132.jpg</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="L14" s="1" t="n"/>
+      <c r="M14" s="1" t="n"/>
+      <c r="N14" s="1" t="n"/>
+      <c r="O14" s="1" t="n"/>
+    </row>
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>porsche-studio</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Porsche Studio </t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>PORSCHE STUDIO</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="n"/>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>This is an authentic reproduction of Porsche’s iconic "Studio Check" automotive upholstery fabric, specifically curated for  Porsche 911 Carrera (964/993 generations), Porsche 928, and Porsche 968</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="n"/>
+      <c r="G15" s="1" t="inlineStr">
+        <is>
+          <t>Porsche Studio Check Grey Fabric | 964 993 928 Restoration Cloth</t>
+        </is>
+      </c>
+      <c r="H15" s="1" t="n"/>
+      <c r="I15" s="1" t="inlineStr">
+        <is>
+          <t>Vintage Authentic reproduction of the classic Porsche Studio Check upholstery fabric</t>
+        </is>
+      </c>
+      <c r="J15" s="1" t="n"/>
+      <c r="K15" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8118.jpg</t>
         </is>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="L15" s="1" t="n"/>
+      <c r="M15" s="1" t="n"/>
+      <c r="N15" s="1" t="n"/>
+      <c r="O15" s="1" t="n"/>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>porsche-tartan</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Porsche Tartan</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>PORSCHE TARTAN</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="n"/>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Introduced in 1975, this legendary pattern was famously optioned on the early Porsche 911 Turbo (930) and the 911SC</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="n"/>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>Porsche Classic Tartan Fabric | 911SC &amp; 930 Turbo Seat Cloth</t>
+        </is>
+      </c>
+      <c r="H16" s="1" t="n"/>
+      <c r="I16" s="1" t="inlineStr">
+        <is>
+          <t>Vintage-style  plaid upholstery cloth for classic Porsche interiors. Durable, period-correct flatwoven check fabric for seats and door cards.</t>
+        </is>
+      </c>
+      <c r="J16" s="1" t="n"/>
+      <c r="K16" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8217.jpg</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="L16" s="1" t="n"/>
+      <c r="M16" s="1" t="n"/>
+      <c r="N16" s="1" t="n"/>
+      <c r="O16" s="1" t="n"/>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>selected-plaid</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Selected Plaid</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>SELETED PLAID</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="n"/>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>Selected plaid for automotive seat upholstery</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="n"/>
+      <c r="G17" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Automotive Plaid for Seat Upholstery </t>
+        </is>
+      </c>
+      <c r="H17" s="1" t="n"/>
+      <c r="I17" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Polyester automtive plaid for seat upholstery </t>
+        </is>
+      </c>
+      <c r="J17" s="1" t="n"/>
+      <c r="K17" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8517.jpg</t>
         </is>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="L17" s="1" t="n"/>
+      <c r="M17" s="1" t="n"/>
+      <c r="N17" s="1" t="n"/>
+      <c r="O17" s="1" t="n"/>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>spirit-of-le-mans</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Spirit of Le Mans</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>SPIRIT OF LE MANS</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="n"/>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>The Spirit of Le Mans (SOLM) Wool Line is a premium, motorsport-inspired tartan collection woven in Scotland and engineered specifically for high-end automotive interiors. 100% premium wool woven in a durable 2/2 twill, featuring a heavy-duty weight of 500 glm (365 gsm). Pre-treated with specialized Soil Resist and Fire Retardant (FR) compliance coatings tailored for automotive safety standards.</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="n"/>
+      <c r="G18" s="1" t="inlineStr">
+        <is>
+          <t>100% Luxury Wool Automotive Fabric | Fire Retardant Tartan</t>
+        </is>
+      </c>
+      <c r="H18" s="1" t="n"/>
+      <c r="I18" s="1" t="inlineStr">
+        <is>
+          <t>Heavyweight wool racing tartan cloth for luxury car interiors. Pre-treated with fire-retardant and soil-resist coatings. Woven in Scotland</t>
+        </is>
+      </c>
+      <c r="J18" s="1" t="n"/>
+      <c r="K18" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA2002.jpg</t>
         </is>
       </c>
+      <c r="L18" s="1" t="n"/>
+      <c r="M18" s="1" t="n"/>
+      <c r="N18" s="1" t="n"/>
+      <c r="O18" s="1" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n"/>
+      <c r="B19" s="1" t="n"/>
+      <c r="C19" s="1" t="n"/>
+      <c r="D19" s="1" t="n"/>
+      <c r="E19" s="1" t="n"/>
+      <c r="F19" s="1" t="n"/>
+      <c r="G19" s="1" t="n"/>
+      <c r="H19" s="1" t="n"/>
+      <c r="I19" s="1" t="n"/>
+      <c r="J19" s="1" t="n"/>
+      <c r="K19" s="1" t="n"/>
+      <c r="L19" s="1" t="n"/>
+      <c r="M19" s="1" t="n"/>
+      <c r="N19" s="1" t="n"/>
+      <c r="O19" s="1" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n"/>
+      <c r="B20" s="1" t="n"/>
+      <c r="C20" s="1" t="n"/>
+      <c r="D20" s="1" t="n"/>
+      <c r="E20" s="1" t="n"/>
+      <c r="F20" s="1" t="n"/>
+      <c r="G20" s="1" t="n"/>
+      <c r="H20" s="1" t="n"/>
+      <c r="I20" s="1" t="n"/>
+      <c r="J20" s="1" t="n"/>
+      <c r="K20" s="1" t="n"/>
+      <c r="L20" s="1" t="n"/>
+      <c r="M20" s="1" t="n"/>
+      <c r="N20" s="1" t="n"/>
+      <c r="O20" s="1" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n"/>
+      <c r="B21" s="1" t="n"/>
+      <c r="C21" s="1" t="n"/>
+      <c r="D21" s="1" t="n"/>
+      <c r="E21" s="1" t="n"/>
+      <c r="F21" s="1" t="n"/>
+      <c r="G21" s="1" t="n"/>
+      <c r="H21" s="1" t="n"/>
+      <c r="I21" s="1" t="n"/>
+      <c r="J21" s="1" t="n"/>
+      <c r="K21" s="1" t="n"/>
+      <c r="L21" s="1" t="n"/>
+      <c r="M21" s="1" t="n"/>
+      <c r="N21" s="1" t="n"/>
+      <c r="O21" s="1" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n"/>
+      <c r="B22" s="1" t="n"/>
+      <c r="C22" s="1" t="n"/>
+      <c r="D22" s="1" t="n"/>
+      <c r="E22" s="1" t="n"/>
+      <c r="F22" s="1" t="n"/>
+      <c r="G22" s="1" t="n"/>
+      <c r="H22" s="1" t="n"/>
+      <c r="I22" s="1" t="n"/>
+      <c r="J22" s="1" t="n"/>
+      <c r="K22" s="1" t="n"/>
+      <c r="L22" s="1" t="n"/>
+      <c r="M22" s="1" t="n"/>
+      <c r="N22" s="1" t="n"/>
+      <c r="O22" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -870,8 +1381,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H86"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <cols>
+    <col width="34.1640625" customWidth="1" min="1" max="1"/>
+    <col width="15.83203125" customWidth="1" min="2" max="2"/>
+    <col width="19.33203125" customWidth="1" min="3" max="3"/>
+    <col width="22.1640625" customWidth="1" min="4" max="4"/>
+    <col width="17.6640625" customWidth="1" min="5" max="5"/>
+    <col width="19.83203125" customWidth="1" min="7" max="7"/>
+    <col width="24.33203125" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -912,6 +1432,2641 @@
       <c r="H1" t="inlineStr">
         <is>
           <t>default_value_ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>bmw-check</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.6mm</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.6mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Wool/Polyester</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>ウール/ポリエステル</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>bmw-m-pattern</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2.0mm</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2.0mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="B9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1">
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Polyester</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ポリエステル</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="B11" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>houndstooth-plaid</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0.8mm</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>0.8mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1">
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1">
+      <c r="B14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
+      <c r="B15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Wool/Polyester</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>ウール/ポリエステル</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="B16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>mercedes-check</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>1.3mm</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1.3mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="B18" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="B20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Wool/Polyester</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>ウール/ポリエステル</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="B21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>mercedes-rodeo</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>1.0mm</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>1.0mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Polyester</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>ポリエステル</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="n">
+        <v>5</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>mercedes-tartan</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>0.8mm</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>0.8mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="n">
+        <v>2</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="n">
+        <v>4</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Wool</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>ウール</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="n">
+        <v>5</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>porsche-check</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>1.3mm</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>1.3mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="n">
+        <v>3</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="n">
+        <v>4</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Wool/Polyester</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>ウール/ポリエステル</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="n">
+        <v>5</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>porsche-herringbone</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>1.2mm</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>1.2mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="n">
+        <v>3</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="n">
+        <v>4</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Wool/Polyester</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>ウール/ポリエステル</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="n">
+        <v>5</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>porsche-madras</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>1.1mm</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>1.1mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="n">
+        <v>4</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Wool/Polyester</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>ウール/ポリエステル</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="n">
+        <v>5</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>porsche-pepita</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>1.1mm</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>1.1mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" t="n">
+        <v>3</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="n">
+        <v>4</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Wool/Polyester</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>ウール/ポリエステル</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" t="n">
+        <v>5</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>porsche-pinstripe</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>1.0mm</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>1.6mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="n">
+        <v>3</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="n">
+        <v>4</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Wool/Polyester</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>ウール/ポリエステル</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="n">
+        <v>5</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>porsche-plaid</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>1.0mm</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>1.0mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="n">
+        <v>2</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" t="n">
+        <v>3</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" t="n">
+        <v>4</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Wool</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>ウール</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" t="n">
+        <v>5</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>porsche-velours-pinstripe</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>1.6mm</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>1.0mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" t="n">
+        <v>3</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" t="n">
+        <v>4</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Wool/Polyester</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>ウール/ポリエステル</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="n">
+        <v>5</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>porsche-studio</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>1.3mm</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>1.3mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" t="n">
+        <v>2</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" t="n">
+        <v>3</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" t="n">
+        <v>4</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Wool/Polyester</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>ウール/ポリエステル</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" t="n">
+        <v>5</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>porsche-tartan</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>1</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>1.3mm</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>1.3mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" t="n">
+        <v>2</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" t="n">
+        <v>3</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" t="n">
+        <v>4</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Wool/Polyester</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>ウール/ポリエステル</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" t="n">
+        <v>5</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>selected-plaid</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>1</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>1.0mm</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>1.0mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" t="n">
+        <v>2</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" t="n">
+        <v>3</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" t="n">
+        <v>4</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Polyester</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>ポリエステル</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" t="n">
+        <v>5</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>spirit-of-le-mans</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>1</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>0.6mm</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>0.6mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" t="n">
+        <v>2</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" t="n">
+        <v>3</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" t="n">
+        <v>4</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Wool</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>ウール</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" t="n">
+        <v>5</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>イギリス</t>
         </is>
       </c>
     </row>
@@ -927,7 +4082,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -963,7 +4118,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1009,7 +4164,18 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q41"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <cols>
+    <col width="20.1640625" customWidth="1" min="3" max="3"/>
+    <col width="36.83203125" customWidth="1" min="5" max="5"/>
+    <col width="21.33203125" customWidth="1" min="6" max="6"/>
+    <col width="35.83203125" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="30.1640625" customWidth="1" min="12" max="13"/>
+    <col width="21.83203125" customWidth="1" min="14" max="14"/>
+    <col width="22.33203125" customWidth="1" min="15" max="15"/>
+    <col width="36.6640625" customWidth="1" min="16" max="16"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1119,6 +4285,11 @@
           <t>FA1836</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>BLACK/GRAY/BROWN</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>/uploads/fabric/BMW Check/FA1836.jpg</t>
@@ -1161,6 +4332,11 @@
           <t>FA5990</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>M PATTERN</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>/uploads/fabric/BMW M Pattern/FA5990.jpg</t>
@@ -1203,6 +4379,11 @@
           <t>FA8765</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>GRAY/WHITE/BROWN</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>/uploads/fabric/Houndstooth Plaid/FA8765.jpg</t>
@@ -1245,6 +4426,11 @@
           <t>FA8475</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>BLACK/BROWN/RED</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>/uploads/fabric/Mercedes Check /FA8475.jpg</t>
@@ -1287,6 +4473,11 @@
           <t>FA8598</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>GRAY/BLACK</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>/uploads/fabric/Mercedes Rodeo/FA8598.jpg</t>
@@ -1329,6 +4520,11 @@
           <t>FA8626</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>BLUE/GRAY</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>/uploads/fabric/Mercedes Tartan/FA8626.jpg</t>
@@ -1371,6 +4567,11 @@
           <t>FA8637</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>GREEN/GRAY/WHITE</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>/uploads/fabric/Mercedes Tartan/FA8637.jpg</t>
@@ -1413,6 +4614,11 @@
           <t>FA8045</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>BLACK/BROWN/YELLOW</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Check/FA8045.jpg</t>
@@ -1455,6 +4661,11 @@
           <t>FA8057</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>BROWN/TAN/GREEN</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Check/FA8057.jpg</t>
@@ -1497,6 +4708,11 @@
           <t>FA8063</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>BLACK/WHITE/RED</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Check/FA8063.jpg</t>
@@ -1539,6 +4755,11 @@
           <t>FA3570</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>BLACK/WHITE</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Herringbone/FA3570.jpg</t>
@@ -1581,6 +4802,11 @@
           <t>FA8326</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>BLUE/WHITE</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Madras/FA8326.jpg</t>
@@ -1623,6 +4849,11 @@
           <t>FA8354</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ORANGE/BROWN</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Madras/FA8354.jpg</t>
@@ -1665,6 +4896,11 @@
           <t>FA8013</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>BLACK/WHITE/ORANGE</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pepita/FA8013.jpg</t>
@@ -1707,6 +4943,11 @@
           <t>FA8026</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>BLACK/WHITE/BLUE</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pepita/FA8026.jpg</t>
@@ -1749,6 +4990,11 @@
           <t>FA8065</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>BLACK/WHITE</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pepita/FA8065.jpg</t>
@@ -1791,6 +5037,11 @@
           <t>FA8074</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>BLACK/WHITE/BEIGE</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pepita/FA8074.jpg</t>
@@ -1833,6 +5084,11 @@
           <t>FA8093</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>BLACK/WHITE/GREEN</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pepita/FA8093.jpg</t>
@@ -1875,6 +5131,11 @@
           <t>FA8094</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>BLACK/WHITE/RED</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pepita/FA8094.jpg</t>
@@ -1917,6 +5178,11 @@
           <t>FA3018</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>BURGUNDY/WHITE</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pinstripe/FA3018.jpg</t>
@@ -1959,6 +5225,11 @@
           <t>FA3055</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>MAROON/WHITE</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pinstripe/FA3055.jpg</t>
@@ -2001,6 +5272,11 @@
           <t>FA3067</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>BLACK/DARK GRAY/GRAY</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pinstripe/FA3067.jpg</t>
@@ -2043,6 +5319,11 @@
           <t>FA3074</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>BLACK/WHITE</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Pinstripe/FA3074.jpg</t>
@@ -2085,6 +5366,11 @@
           <t>FA8525</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>BLUE/BLACK/WHITE/RED</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Plaid/FA8525.jpg</t>
@@ -2119,7 +5405,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>porsche-script</t>
+          <t>porsche-pinstripe</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2127,14 +5413,19 @@
           <t>FA3132</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>GRAY/BLUE</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Script/FA3132.jpg</t>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3132.jpg</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Script/FA3132.jpg</t>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3132.jpg</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2144,7 +5435,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Script/FA3132.jpg</t>
+          <t>/uploads/fabric/Porsche Pinstripe/FA3132.jpg</t>
         </is>
       </c>
     </row>
@@ -2161,7 +5452,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>porsche-script</t>
+          <t>porsche-velours-pinstripe</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2169,14 +5460,19 @@
           <t>FA3217</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>BLACK/RED</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Script/FA3217.jpg</t>
+          <t>/uploads/fabric/Porsche Velcours Pinstripe/FA3217.jpg</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Script/FA3217.jpg</t>
+          <t>/uploads/fabric/Porsche Velcours Pinstripe/FA3217.jpg</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2186,7 +5482,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Script/FA3217.jpg</t>
+          <t>/uploads/fabric/Porsche Velcours Pinstripe/FA3217.jpg</t>
         </is>
       </c>
     </row>
@@ -2203,7 +5499,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>porsche-script</t>
+          <t>porsche-velours-pinstripe</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2211,14 +5507,19 @@
           <t>FA3258</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>BROWN/WHITE</t>
+        </is>
+      </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Script/FA3258.jpg</t>
+          <t>/uploads/fabric/Porsche Velcours Pinstripe/FA3258.jpg</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Script/FA3258.jpg</t>
+          <t>/uploads/fabric/Porsche Velcours Pinstripe/FA3258.jpg</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2228,7 +5529,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Script/FA3258.jpg</t>
+          <t>/uploads/fabric/Porsche Velcours Pinstripe/FA3258.jpg</t>
         </is>
       </c>
     </row>
@@ -2245,7 +5546,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>porsche-script</t>
+          <t>porsche-velours-pinstripe</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2253,14 +5554,19 @@
           <t>FA3272</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>GRAY/WHITE</t>
+        </is>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Script/FA3272.jpg</t>
+          <t>/uploads/fabric/Porsche Velcours Pinstripe/FA3272.jpg</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Script/FA3272.jpg</t>
+          <t>/uploads/fabric/Porsche Velcours Pinstripe/FA3272.jpg</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2270,7 +5576,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Porsche Script/FA3272.jpg</t>
+          <t>/uploads/fabric/Porsche Velcours Pinstripe/FA3272.jpg</t>
         </is>
       </c>
     </row>
@@ -2295,6 +5601,11 @@
           <t>FA8118</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>RED/MAROON</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Studio /FA8118.jpg</t>
@@ -2337,6 +5648,11 @@
           <t>FA8128</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>NAVY/BLUE/BLACK</t>
+        </is>
+      </c>
       <c r="H31" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Studio /FA8128.jpg</t>
@@ -2379,6 +5695,11 @@
           <t>FA8165</t>
         </is>
       </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>GRAY</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Studio /FA8165.jpg</t>
@@ -2421,6 +5742,11 @@
           <t>FA8166</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>GRAY</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Studio /FA8166.jpg</t>
@@ -2463,6 +5789,11 @@
           <t>FA8217</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>BLUE/RED/BLACK</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Tartan/FA8217 McLaughli.jpg</t>
@@ -2505,6 +5836,11 @@
           <t>FA8237</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>NAVY/BLUE/BLACK</t>
+        </is>
+      </c>
       <c r="H35" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Tartan/FA8237 Black Watch.jpg</t>
@@ -2547,6 +5883,11 @@
           <t>FA8271</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>GRAY/BLUE/WHITE</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
           <t>/uploads/fabric/Porsche Tartan/FA8271 Mackenzie.jpg</t>
@@ -2589,6 +5930,11 @@
           <t>FA8517</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>BLACK/RED/BLUE</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>/uploads/fabric/Selected Plaid/FA8517.jpg</t>
@@ -2631,6 +5977,11 @@
           <t>FA8553</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>BLUE/NAVY/ORANGE</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>/uploads/fabric/Selected Plaid/FA8553.jpg</t>
@@ -2673,6 +6024,11 @@
           <t>FA2002</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>BLUE/NAVY/RED</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>/uploads/fabric/Spirit of Le Mans/FA2002.jpg</t>
@@ -2715,6 +6071,11 @@
           <t>FA2202</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>BLUE/ORANGE/NAVY</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
           <t>/uploads/fabric/Spirit of Le Mans/FA2202.jpg</t>
@@ -2755,6 +6116,11 @@
       <c r="D41" t="inlineStr">
         <is>
           <t>FA2729</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>BLUE/BLACK/RED</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2790,7 +6156,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2836,7 +6202,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2892,7 +6258,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E41"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>

<commit_message>
Update fabric product slugs and velours cover
</commit_message>
<xml_diff>
--- a/data/import/fabric/fabric.xlsx
+++ b/data/import/fabric/fabric.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="320" yWindow="780" windowWidth="33900" windowHeight="19660" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="300" yWindow="780" windowWidth="33900" windowHeight="19660" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="product_types" sheetId="1" state="visible" r:id="rId1"/>
@@ -1114,7 +1114,7 @@
       <c r="J14" s="1" t="n"/>
       <c r="K14" s="1" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Cover/FA3132.jpg</t>
+          <t>/uploads/fabric/Cover/FA3217.jpg</t>
         </is>
       </c>
       <c r="L14" s="1" t="n"/>
@@ -1471,6 +1471,11 @@
       </c>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>bmw-check</t>
+        </is>
+      </c>
       <c r="B3" t="n">
         <v>2</v>
       </c>
@@ -1501,6 +1506,11 @@
       </c>
     </row>
     <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>bmw-check</t>
+        </is>
+      </c>
       <c r="B4" t="n">
         <v>3</v>
       </c>
@@ -1531,6 +1541,11 @@
       </c>
     </row>
     <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>bmw-check</t>
+        </is>
+      </c>
       <c r="B5" t="n">
         <v>4</v>
       </c>
@@ -1561,6 +1576,11 @@
       </c>
     </row>
     <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>bmw-check</t>
+        </is>
+      </c>
       <c r="B6" t="n">
         <v>5</v>
       </c>
@@ -1626,6 +1646,11 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>bmw-m-pattern</t>
+        </is>
+      </c>
       <c r="B8" t="n">
         <v>2</v>
       </c>
@@ -1656,6 +1681,11 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>bmw-m-pattern</t>
+        </is>
+      </c>
       <c r="B9" t="n">
         <v>3</v>
       </c>
@@ -1686,6 +1716,11 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>bmw-m-pattern</t>
+        </is>
+      </c>
       <c r="B10" t="n">
         <v>4</v>
       </c>
@@ -1716,6 +1751,11 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>bmw-m-pattern</t>
+        </is>
+      </c>
       <c r="B11" t="n">
         <v>5</v>
       </c>
@@ -1781,6 +1821,11 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>houndstooth-plaid</t>
+        </is>
+      </c>
       <c r="B13" t="n">
         <v>2</v>
       </c>
@@ -1811,6 +1856,11 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>houndstooth-plaid</t>
+        </is>
+      </c>
       <c r="B14" t="n">
         <v>3</v>
       </c>
@@ -1841,6 +1891,11 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>houndstooth-plaid</t>
+        </is>
+      </c>
       <c r="B15" t="n">
         <v>4</v>
       </c>
@@ -1871,6 +1926,11 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>houndstooth-plaid</t>
+        </is>
+      </c>
       <c r="B16" t="n">
         <v>5</v>
       </c>
@@ -1936,6 +1996,11 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>mercedes-check</t>
+        </is>
+      </c>
       <c r="B18" t="n">
         <v>2</v>
       </c>
@@ -1966,6 +2031,11 @@
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>mercedes-check</t>
+        </is>
+      </c>
       <c r="B19" t="n">
         <v>3</v>
       </c>
@@ -1996,6 +2066,11 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>mercedes-check</t>
+        </is>
+      </c>
       <c r="B20" t="n">
         <v>4</v>
       </c>
@@ -2026,6 +2101,11 @@
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>mercedes-check</t>
+        </is>
+      </c>
       <c r="B21" t="n">
         <v>5</v>
       </c>
@@ -2091,6 +2171,11 @@
       </c>
     </row>
     <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>mercedes-rodeo</t>
+        </is>
+      </c>
       <c r="B23" t="n">
         <v>2</v>
       </c>
@@ -2121,6 +2206,11 @@
       </c>
     </row>
     <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>mercedes-rodeo</t>
+        </is>
+      </c>
       <c r="B24" t="n">
         <v>3</v>
       </c>
@@ -2151,6 +2241,11 @@
       </c>
     </row>
     <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>mercedes-rodeo</t>
+        </is>
+      </c>
       <c r="B25" t="n">
         <v>4</v>
       </c>
@@ -2181,6 +2276,11 @@
       </c>
     </row>
     <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>mercedes-rodeo</t>
+        </is>
+      </c>
       <c r="B26" t="n">
         <v>5</v>
       </c>
@@ -2246,6 +2346,11 @@
       </c>
     </row>
     <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>mercedes-tartan</t>
+        </is>
+      </c>
       <c r="B28" t="n">
         <v>2</v>
       </c>
@@ -2276,6 +2381,11 @@
       </c>
     </row>
     <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>mercedes-tartan</t>
+        </is>
+      </c>
       <c r="B29" t="n">
         <v>3</v>
       </c>
@@ -2306,6 +2416,11 @@
       </c>
     </row>
     <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>mercedes-tartan</t>
+        </is>
+      </c>
       <c r="B30" t="n">
         <v>4</v>
       </c>
@@ -2336,6 +2451,11 @@
       </c>
     </row>
     <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>mercedes-tartan</t>
+        </is>
+      </c>
       <c r="B31" t="n">
         <v>5</v>
       </c>
@@ -2401,6 +2521,11 @@
       </c>
     </row>
     <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>porsche-check</t>
+        </is>
+      </c>
       <c r="B33" t="n">
         <v>2</v>
       </c>
@@ -2431,6 +2556,11 @@
       </c>
     </row>
     <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>porsche-check</t>
+        </is>
+      </c>
       <c r="B34" t="n">
         <v>3</v>
       </c>
@@ -2461,6 +2591,11 @@
       </c>
     </row>
     <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>porsche-check</t>
+        </is>
+      </c>
       <c r="B35" t="n">
         <v>4</v>
       </c>
@@ -2491,6 +2626,11 @@
       </c>
     </row>
     <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>porsche-check</t>
+        </is>
+      </c>
       <c r="B36" t="n">
         <v>5</v>
       </c>
@@ -2556,6 +2696,11 @@
       </c>
     </row>
     <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>porsche-herringbone</t>
+        </is>
+      </c>
       <c r="B38" t="n">
         <v>2</v>
       </c>
@@ -2586,6 +2731,11 @@
       </c>
     </row>
     <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>porsche-herringbone</t>
+        </is>
+      </c>
       <c r="B39" t="n">
         <v>3</v>
       </c>
@@ -2616,6 +2766,11 @@
       </c>
     </row>
     <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>porsche-herringbone</t>
+        </is>
+      </c>
       <c r="B40" t="n">
         <v>4</v>
       </c>
@@ -2646,6 +2801,11 @@
       </c>
     </row>
     <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>porsche-herringbone</t>
+        </is>
+      </c>
       <c r="B41" t="n">
         <v>5</v>
       </c>
@@ -2711,6 +2871,11 @@
       </c>
     </row>
     <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>porsche-madras</t>
+        </is>
+      </c>
       <c r="B43" t="n">
         <v>2</v>
       </c>
@@ -2741,6 +2906,11 @@
       </c>
     </row>
     <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>porsche-madras</t>
+        </is>
+      </c>
       <c r="B44" t="n">
         <v>3</v>
       </c>
@@ -2771,6 +2941,11 @@
       </c>
     </row>
     <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>porsche-madras</t>
+        </is>
+      </c>
       <c r="B45" t="n">
         <v>4</v>
       </c>
@@ -2801,6 +2976,11 @@
       </c>
     </row>
     <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>porsche-madras</t>
+        </is>
+      </c>
       <c r="B46" t="n">
         <v>5</v>
       </c>
@@ -2866,6 +3046,11 @@
       </c>
     </row>
     <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>porsche-pepita</t>
+        </is>
+      </c>
       <c r="B48" t="n">
         <v>2</v>
       </c>
@@ -2896,6 +3081,11 @@
       </c>
     </row>
     <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>porsche-pepita</t>
+        </is>
+      </c>
       <c r="B49" t="n">
         <v>3</v>
       </c>
@@ -2926,6 +3116,11 @@
       </c>
     </row>
     <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>porsche-pepita</t>
+        </is>
+      </c>
       <c r="B50" t="n">
         <v>4</v>
       </c>
@@ -2956,6 +3151,11 @@
       </c>
     </row>
     <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>porsche-pepita</t>
+        </is>
+      </c>
       <c r="B51" t="n">
         <v>5</v>
       </c>
@@ -3021,6 +3221,11 @@
       </c>
     </row>
     <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>porsche-pinstripe</t>
+        </is>
+      </c>
       <c r="B53" t="n">
         <v>2</v>
       </c>
@@ -3051,6 +3256,11 @@
       </c>
     </row>
     <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>porsche-pinstripe</t>
+        </is>
+      </c>
       <c r="B54" t="n">
         <v>3</v>
       </c>
@@ -3081,6 +3291,11 @@
       </c>
     </row>
     <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>porsche-pinstripe</t>
+        </is>
+      </c>
       <c r="B55" t="n">
         <v>4</v>
       </c>
@@ -3111,6 +3326,11 @@
       </c>
     </row>
     <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>porsche-pinstripe</t>
+        </is>
+      </c>
       <c r="B56" t="n">
         <v>5</v>
       </c>
@@ -3176,6 +3396,11 @@
       </c>
     </row>
     <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>porsche-plaid</t>
+        </is>
+      </c>
       <c r="B58" t="n">
         <v>2</v>
       </c>
@@ -3206,6 +3431,11 @@
       </c>
     </row>
     <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>porsche-plaid</t>
+        </is>
+      </c>
       <c r="B59" t="n">
         <v>3</v>
       </c>
@@ -3236,6 +3466,11 @@
       </c>
     </row>
     <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>porsche-plaid</t>
+        </is>
+      </c>
       <c r="B60" t="n">
         <v>4</v>
       </c>
@@ -3266,6 +3501,11 @@
       </c>
     </row>
     <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>porsche-plaid</t>
+        </is>
+      </c>
       <c r="B61" t="n">
         <v>5</v>
       </c>
@@ -3331,6 +3571,11 @@
       </c>
     </row>
     <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>porsche-velours-pinstripe</t>
+        </is>
+      </c>
       <c r="B63" t="n">
         <v>2</v>
       </c>
@@ -3361,6 +3606,11 @@
       </c>
     </row>
     <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>porsche-velours-pinstripe</t>
+        </is>
+      </c>
       <c r="B64" t="n">
         <v>3</v>
       </c>
@@ -3391,6 +3641,11 @@
       </c>
     </row>
     <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>porsche-velours-pinstripe</t>
+        </is>
+      </c>
       <c r="B65" t="n">
         <v>4</v>
       </c>
@@ -3421,6 +3676,11 @@
       </c>
     </row>
     <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>porsche-velours-pinstripe</t>
+        </is>
+      </c>
       <c r="B66" t="n">
         <v>5</v>
       </c>
@@ -3486,6 +3746,11 @@
       </c>
     </row>
     <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>porsche-studio</t>
+        </is>
+      </c>
       <c r="B68" t="n">
         <v>2</v>
       </c>
@@ -3516,6 +3781,11 @@
       </c>
     </row>
     <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>porsche-studio</t>
+        </is>
+      </c>
       <c r="B69" t="n">
         <v>3</v>
       </c>
@@ -3546,6 +3816,11 @@
       </c>
     </row>
     <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>porsche-studio</t>
+        </is>
+      </c>
       <c r="B70" t="n">
         <v>4</v>
       </c>
@@ -3576,6 +3851,11 @@
       </c>
     </row>
     <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>porsche-studio</t>
+        </is>
+      </c>
       <c r="B71" t="n">
         <v>5</v>
       </c>
@@ -3641,6 +3921,11 @@
       </c>
     </row>
     <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>porsche-tartan</t>
+        </is>
+      </c>
       <c r="B73" t="n">
         <v>2</v>
       </c>
@@ -3671,6 +3956,11 @@
       </c>
     </row>
     <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>porsche-tartan</t>
+        </is>
+      </c>
       <c r="B74" t="n">
         <v>3</v>
       </c>
@@ -3701,6 +3991,11 @@
       </c>
     </row>
     <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>porsche-tartan</t>
+        </is>
+      </c>
       <c r="B75" t="n">
         <v>4</v>
       </c>
@@ -3731,6 +4026,11 @@
       </c>
     </row>
     <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>porsche-tartan</t>
+        </is>
+      </c>
       <c r="B76" t="n">
         <v>5</v>
       </c>
@@ -3796,6 +4096,11 @@
       </c>
     </row>
     <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>selected-plaid</t>
+        </is>
+      </c>
       <c r="B78" t="n">
         <v>2</v>
       </c>
@@ -3826,6 +4131,11 @@
       </c>
     </row>
     <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>selected-plaid</t>
+        </is>
+      </c>
       <c r="B79" t="n">
         <v>3</v>
       </c>
@@ -3856,6 +4166,11 @@
       </c>
     </row>
     <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>selected-plaid</t>
+        </is>
+      </c>
       <c r="B80" t="n">
         <v>4</v>
       </c>
@@ -3886,6 +4201,11 @@
       </c>
     </row>
     <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>selected-plaid</t>
+        </is>
+      </c>
       <c r="B81" t="n">
         <v>5</v>
       </c>
@@ -3951,6 +4271,11 @@
       </c>
     </row>
     <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>spirit-of-le-mans</t>
+        </is>
+      </c>
       <c r="B83" t="n">
         <v>2</v>
       </c>
@@ -3981,6 +4306,11 @@
       </c>
     </row>
     <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>spirit-of-le-mans</t>
+        </is>
+      </c>
       <c r="B84" t="n">
         <v>3</v>
       </c>
@@ -4011,6 +4341,11 @@
       </c>
     </row>
     <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>spirit-of-le-mans</t>
+        </is>
+      </c>
       <c r="B85" t="n">
         <v>4</v>
       </c>
@@ -4041,6 +4376,11 @@
       </c>
     </row>
     <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>spirit-of-le-mans</t>
+        </is>
+      </c>
       <c r="B86" t="n">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
Update generated material catalog
</commit_message>
<xml_diff>
--- a/data/import/fabric/fabric.xlsx
+++ b/data/import/fabric/fabric.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="300" yWindow="780" windowWidth="33900" windowHeight="19660" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="300" yWindow="780" windowWidth="33900" windowHeight="19660" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="product_types" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="product_type_specs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="product_type_certifications" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="product_type_maintenance" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="skus" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="sku_specs" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="product_type_downloads" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="sku_case_gallery" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="product_types" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="product_type_specs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="product_type_certifications" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="product_type_maintenance" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="skus" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sku_specs" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="product_type_downloads" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sku_case_gallery" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -461,11 +461,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O22"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
-    <col width="24.33203125" customWidth="1" min="3" max="3"/>
+    <col width="25.6640625" customWidth="1" min="3" max="3"/>
     <col width="17.83203125" customWidth="1" min="4" max="4"/>
     <col width="47.33203125" customWidth="1" min="5" max="5"/>
     <col width="18.6640625" customWidth="1" min="6" max="6"/>
@@ -473,6 +473,7 @@
     <col width="17.33203125" customWidth="1" min="8" max="8"/>
     <col width="38.5" customWidth="1" min="9" max="9"/>
     <col width="21.83203125" customWidth="1" min="10" max="10"/>
+    <col width="44.1640625" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -553,25 +554,41 @@
           <t>BMW CHECK</t>
         </is>
       </c>
-      <c r="D2" s="1" t="n"/>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>BMW チェック</t>
+        </is>
+      </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Classic Scottish square pattern for BMW Isetta</t>
         </is>
       </c>
-      <c r="F2" s="1" t="n"/>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>BMWイセッタ向けのクラシックなスコットランドスクエアパターン。</t>
+        </is>
+      </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
           <t>BMW Isetta Classic Tartan Seat Upholstery Fabric</t>
         </is>
       </c>
-      <c r="H2" s="1" t="n"/>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>BMWイセッタ クラシックタータン シート張り地</t>
+        </is>
+      </c>
       <c r="I2" s="1" t="inlineStr">
         <is>
           <t>Authentic flatwoven green Scottish square fabric for BMW Isetta restoration (models up to 1958).Exact OEM match pattern. Inquire for rolls.</t>
         </is>
       </c>
-      <c r="J2" s="1" t="n"/>
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>BMWイセッタ（1958年以前モデル）レストア用の本格的なフラットウィーブングリーンスコットランドスクエアファブリック。純正OEMマッチパターン。ロールでのお問い合わせ承ります。</t>
+        </is>
+      </c>
       <c r="K2" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA1836.jpg</t>
@@ -598,25 +615,41 @@
           <t>BMW M PATTERN</t>
         </is>
       </c>
-      <c r="D3" s="1" t="n"/>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>BMW M パターン</t>
+        </is>
+      </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
           <t>The M-Stripe seat cloth is a  replica of the original material used in the prototype M8.</t>
         </is>
       </c>
-      <c r="F3" s="1" t="n"/>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Mストライプシートクロスは、プロトタイプM8に使用されたオリジナル素材のレプリカです。</t>
+        </is>
+      </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
           <t>BMW Seat Fabric with Foam</t>
         </is>
       </c>
-      <c r="H3" s="1" t="n"/>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>BMW Mシートファブリック（フォーム付き）</t>
+        </is>
+      </c>
       <c r="I3" s="1" t="inlineStr">
         <is>
           <t>Premium reproduction of the iconic M Jahre M-Stripe seat fabric. A replica of the ultra-rare material found in the legendary M8 Prototype cabin.</t>
         </is>
       </c>
-      <c r="J3" s="1" t="n"/>
+      <c r="J3" s="1" t="inlineStr">
+        <is>
+          <t>象徴的なMヤーレMストライプシート生地のプレミアム復刻版。伝説のM8プロトタイプキャビンに使用された超希少素材のレプリカ。</t>
+        </is>
+      </c>
       <c r="K3" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA5990.jpg</t>
@@ -643,25 +676,41 @@
           <t>HOUNDSTOOTH PLAID</t>
         </is>
       </c>
-      <c r="D4" s="1" t="n"/>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>ハウンドトゥース プレイド</t>
+        </is>
+      </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
           <t>This textile features an intricate houndstooth-based Glen plaid layout blended with Scottish Squares for seat upholstery</t>
         </is>
       </c>
-      <c r="F4" s="1" t="n"/>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>千鳥格子ベースのグレンチェックにスコティッシュスクエアを組み合わせた複雑なレイアウトのシート張り地。</t>
+        </is>
+      </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
           <t>Houndstooth based Glen plaid with Tartan for Seat Upholstery</t>
         </is>
       </c>
-      <c r="H4" s="1" t="n"/>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>千鳥格子ベース グレンチェック×タータン シート張り地</t>
+        </is>
+      </c>
       <c r="I4" s="1" t="inlineStr">
         <is>
           <t>Premium automotive seat upholstery featuring an intricate houndstooth-based Glen plaid layout blended with Scottish squares. Perfect for vintage car restoration.</t>
         </is>
       </c>
-      <c r="J4" s="1" t="n"/>
+      <c r="J4" s="1" t="inlineStr">
+        <is>
+          <t>千鳥格子ベースのグレンチェックレイアウトにスコティッシュスクエアを融合させたプレミアム自動車用シート張り地。ヴィンテージカーレストアに最適。</t>
+        </is>
+      </c>
       <c r="K4" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8765.jpg</t>
@@ -688,25 +737,41 @@
           <t xml:space="preserve">MERCEDES CHECK </t>
         </is>
       </c>
-      <c r="D5" s="1" t="n"/>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>メルセデス チェック</t>
+        </is>
+      </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
           <t>This premium, original-specification automotive interior textile is an authentic factory-match reproduction of the classic first-generation Mercedes-Benz W460 G-Klasse (G-Wagon)</t>
         </is>
       </c>
-      <c r="F5" s="1" t="n"/>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>初代メルセデス・ベンツ W460 Gクラス（G-Wagon）のクラシックな内装を忠実に再現した、プレミアムな純正スペックの自動車用内装テキスタイル。</t>
+        </is>
+      </c>
       <c r="G5" s="1" t="inlineStr">
         <is>
           <t>Vintage Mercedes G-Wagon Seat Upholstery Fabric</t>
         </is>
       </c>
-      <c r="H5" s="1" t="n"/>
+      <c r="H5" s="1" t="inlineStr">
+        <is>
+          <t>ヴィンテージ メルセデス G-Wagon シート張り地</t>
+        </is>
+      </c>
       <c r="I5" s="1" t="inlineStr">
         <is>
           <t>Authentic 1980s Mercedes W460 G-class seat upholstery fabric. Heavy-duty flatwoven Panamabond square design in Beige Black</t>
         </is>
       </c>
-      <c r="J5" s="1" t="n"/>
+      <c r="J5" s="1" t="inlineStr">
+        <is>
+          <t>1980年代メルセデス W460 Gクラス純正シート張り地。ベージュブラックのヘビーデューティーフラットウィーブンパナマボンドスクエアデザイン。</t>
+        </is>
+      </c>
       <c r="K5" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8475.jpg</t>
@@ -733,25 +798,41 @@
           <t>MERCEDES RODEO</t>
         </is>
       </c>
-      <c r="D6" s="1" t="n"/>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>メルセデス ロデオ</t>
+        </is>
+      </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
           <t>This premium, original-specification automotive interior textile is an authentic factory-match reproduction of the late 1980's Mercedes-Benz G-Klasse. The same pattern is used in 2025 G550 'Stronger Than the 1980s" Special Edition</t>
         </is>
       </c>
-      <c r="F6" s="1" t="n"/>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>1980年代後半のメルセデス・ベンツ Gクラスを忠実に再現したプレミアムな純正スペックファブリック。2025年G550「Stronger Than the 1980s」特別仕様車と同パターン。</t>
+        </is>
+      </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
           <t>Mercedes G-Wagon 'Stronger Than the 1980s'  Seat Fabric</t>
         </is>
       </c>
-      <c r="H6" s="1" t="n"/>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>メルセデス G-Wagon「Stronger Than the 1980s」シート生地</t>
+        </is>
+      </c>
       <c r="I6" s="1" t="inlineStr">
         <is>
           <t>Get the look of the limited edition G550 Stronger Than the 1980s cabin. Authentic Mercedes Rodeo Grey-Black cube upholstery fabric</t>
         </is>
       </c>
-      <c r="J6" s="1" t="n"/>
+      <c r="J6" s="1" t="inlineStr">
+        <is>
+          <t>限定版G550 Stronger Than the 1980sキャビンの外観を実現。本格的なメルセデスロデオグレーブラックキューブ張り地。</t>
+        </is>
+      </c>
       <c r="K6" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8598.jpg</t>
@@ -778,25 +859,41 @@
           <t>MERCEDES TARTAN</t>
         </is>
       </c>
-      <c r="D7" s="1" t="n"/>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>メルセデス タータン</t>
+        </is>
+      </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Woven from 100% pure wool, this elite fabric is engineered exclusively for interior restoration of the legendary Mercedes-Benz W198 300SL Gullwing</t>
         </is>
       </c>
-      <c r="F7" s="1" t="n"/>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>伝説のメルセデス・ベンツ W198 300SL ガルウィングの内装レストア専用に織られた、100%ピュアウールのエリートファブリック。</t>
+        </is>
+      </c>
       <c r="G7" s="1" t="inlineStr">
         <is>
           <t>Mercedes W198 300SL Gullwing 100% Wool Fabric</t>
         </is>
       </c>
-      <c r="H7" s="1" t="n"/>
+      <c r="H7" s="1" t="inlineStr">
+        <is>
+          <t>メルセデス W198 300SL ガルウィング 100%ウール生地</t>
+        </is>
+      </c>
       <c r="I7" s="1" t="inlineStr">
         <is>
           <t>Authentic 100% wool 1954-1963 Mercedes-Benz W198 300SL Gullwing seat fabric. Factory-match blue/grey Scottish square tartan</t>
         </is>
       </c>
-      <c r="J7" s="1" t="n"/>
+      <c r="J7" s="1" t="inlineStr">
+        <is>
+          <t>1954-1963年メルセデス・ベンツ W198 300SLガルウィング用本格的な100%ウールシート生地。純正マッチのブルー/グレースコティッシュスクエアタータン。</t>
+        </is>
+      </c>
       <c r="K7" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8626.jpg</t>
@@ -823,25 +920,41 @@
           <t>PORSCHE CHECK</t>
         </is>
       </c>
-      <c r="D8" s="1" t="n"/>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>ポルシェ チェック</t>
+        </is>
+      </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
           <t>Classic pattern Porsche upholstery fabric</t>
         </is>
       </c>
-      <c r="F8" s="1" t="n"/>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>クラシックパターンのポルシェ張り地。</t>
+        </is>
+      </c>
       <c r="G8" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Vintage Porsche Seating Upholstery Fabric </t>
         </is>
       </c>
-      <c r="H8" s="1" t="n"/>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>ヴィンテージ ポルシェ シート張り地</t>
+        </is>
+      </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Vintage Porsche Seating Upholstery Fabric </t>
         </is>
       </c>
-      <c r="J8" s="1" t="n"/>
+      <c r="J8" s="1" t="inlineStr">
+        <is>
+          <t>ヴィンテージポルシェシート張り地。</t>
+        </is>
+      </c>
       <c r="K8" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8045.jpg</t>
@@ -868,25 +981,41 @@
           <t>PORSCHE HERRINGBONE</t>
         </is>
       </c>
-      <c r="D9" s="1" t="n"/>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>ポルシェ ヘリンボーン</t>
+        </is>
+      </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
           <t>This authentic, OEM-specification automotive seating textile is an exact factory-match reproduction for the upholstery of Porsche 924</t>
         </is>
       </c>
-      <c r="F9" s="1" t="n"/>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>ポルシェ924の張り地を忠実に再現した、本格的なOEMスペックの自動車用シートテキスタイル。</t>
+        </is>
+      </c>
       <c r="G9" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Vintage Porsche Seating Upholstery Fabric Herringbone </t>
         </is>
       </c>
-      <c r="H9" s="1" t="n"/>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>ヴィンテージ ポルシェ ヘリンボーン シート張り地</t>
+        </is>
+      </c>
       <c r="I9" s="1" t="inlineStr">
         <is>
           <t>Authentic 1978 Porsche 924 seat upholstery fabric. Premium factory-match Beige Cream Black herringbone textile</t>
         </is>
       </c>
-      <c r="J9" s="1" t="n"/>
+      <c r="J9" s="1" t="inlineStr">
+        <is>
+          <t>1978年ポルシェ924純正シート張り地。ベージュクリームブラックのヘリンボーンテキスタイル、プレミアムな純正マッチ復刻版。</t>
+        </is>
+      </c>
       <c r="K9" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA3570.jpg</t>
@@ -913,25 +1042,41 @@
           <t>PORSCHE MADRAS</t>
         </is>
       </c>
-      <c r="D10" s="1" t="n"/>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>ポルシェ マドラス</t>
+        </is>
+      </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
           <t>This is the heritage seat upholstery fabric originally offered by Stuttgart as an exclusive cabin option between 1972 and 1975 used in early G-Model Porsche 911s (including the 911T, E, S, and early Carrera).</t>
         </is>
       </c>
-      <c r="F10" s="1" t="n"/>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>1972年から1975年にかけてシュトゥットガルトが限定キャビンオプションとして提供した、ヘリテージシート張り地。アーリーGモデル ポルシェ911（911T、E、S、アーリーカレラ）に採用。</t>
+        </is>
+      </c>
       <c r="G10" s="1" t="inlineStr">
         <is>
           <t>Porsche 911 Madras Seat Upholstery Fabric</t>
         </is>
       </c>
-      <c r="H10" s="1" t="n"/>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>ポルシェ911 マドラス シート張り地</t>
+        </is>
+      </c>
       <c r="I10" s="1" t="inlineStr">
         <is>
           <t>Authentic 1972-1975 Porsche 911 Madras seat fabric. Premium factory-match windowpane plaid for vintage F-Model &amp; G-Model Carrera restorations</t>
         </is>
       </c>
-      <c r="J10" s="1" t="n"/>
+      <c r="J10" s="1" t="inlineStr">
+        <is>
+          <t>1972-1975年ポルシェ911マドラス純正シート生地。ヴィンテージFモデル＆Gモデルカレラレストア向けプレミアム純正マッチウィンドウペーンプレイド。</t>
+        </is>
+      </c>
       <c r="K10" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8326.jpg</t>
@@ -958,25 +1103,41 @@
           <t>PORSCHE PEPITA</t>
         </is>
       </c>
-      <c r="D11" s="1" t="n"/>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>ポルシェ ペピータ</t>
+        </is>
+      </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
           <t>Porsche Pepita is arguably the most famous, style-defining interior textile in sports car history. Officially introduced in 1965 for the original 911, Pepita originated as a special-request option for late-model Porsche 356 classics in the early 1960s.</t>
         </is>
       </c>
-      <c r="F11" s="1" t="n"/>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>スポーツカーの歴史上最も有名でスタイルを定義した内装テキスタイル。1965年にオリジナル911向けに正式導入され、1960年代初頭の後期ポルシェ356クラシックの特別リクエストオプションとして誕生。</t>
+        </is>
+      </c>
       <c r="G11" s="1" t="inlineStr">
         <is>
           <t>Porsche Classic Pepita Fabric | Heritage Design Seat Upholstery</t>
         </is>
       </c>
-      <c r="H11" s="1" t="n"/>
+      <c r="H11" s="1" t="inlineStr">
+        <is>
+          <t>ポルシェ クラシック ペピータ生地 | ヘリテージデザイン シート張り地</t>
+        </is>
+      </c>
       <c r="I11" s="1" t="inlineStr">
         <is>
           <t>Authentic black &amp; white Porsche Pepita seat fabric. Premium factory-match pattern for classic 911 restorations and modern Heritage Design upgrades. More colors available.</t>
         </is>
       </c>
-      <c r="J11" s="1" t="n"/>
+      <c r="J11" s="1" t="inlineStr">
+        <is>
+          <t>本格的なブラック＆ホワイトのポルシェペピータシート生地。クラシック911レストアおよびモダンヘリテージデザインアップグレード向けプレミアム純正マッチパターン。その他カラーも承ります。</t>
+        </is>
+      </c>
       <c r="K11" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8013.jpg</t>
@@ -1003,25 +1164,41 @@
           <t>PORSCHE PINSTRIPE</t>
         </is>
       </c>
-      <c r="D12" s="1" t="n"/>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>ポルシェ ピンストライプ</t>
+        </is>
+      </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Porsche Pinstripe is a highly sophisticated, business-suit-inspired executive textile that defined the interiors of late-1970s and 1980s Porsche sports cars. It became a staple option across the air-cooled 911 (G-Model) series and the entire front-engine transaxle family (924, 944, and 928)</t>
         </is>
       </c>
-      <c r="F12" s="1" t="n"/>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>1970年代後半から1980年代のポルシェスポーツカーの内装を定義した、ビジネススーツに着想を得た非常に洗練されたエグゼクティブテキスタイル。空冷911（Gモデル）シリーズとフロントエンジントランスアクスルファミリー（924、944、928）全体で定番オプションに。</t>
+        </is>
+      </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
           <t>Vintage Porsche Pinstripe Seat Upholstery Fabric</t>
         </is>
       </c>
-      <c r="H12" s="1" t="n"/>
+      <c r="H12" s="1" t="inlineStr">
+        <is>
+          <t>ヴィンテージ ポルシェ ピンストライプ シート張り地</t>
+        </is>
+      </c>
       <c r="I12" s="1" t="inlineStr">
         <is>
           <t>Authentic 1977-1990 Porsche Pinstripe seat fabric. Premium factory-match flannel for classic 911, 924, 928, and 944 cabin restoration.</t>
         </is>
       </c>
-      <c r="J12" s="1" t="n"/>
+      <c r="J12" s="1" t="inlineStr">
+        <is>
+          <t>1977-1990年ポルシェピンストライプ純正シート生地。クラシック911、924、928、944キャビンレストア向けプレミアム純正マッチフランネル。</t>
+        </is>
+      </c>
       <c r="K12" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA3018.jpg</t>
@@ -1048,25 +1225,41 @@
           <t>PORSCHE PLAID</t>
         </is>
       </c>
-      <c r="D13" s="1" t="n"/>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>ポルシェ プレイド</t>
+        </is>
+      </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
           <t>This is a premium 100% wool flatwoven plaid fabric replicated for the 1973 Porsche 911 RSR</t>
         </is>
       </c>
-      <c r="F13" s="1" t="n"/>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>1973年ポルシェ911 RSR向けに再現された、プレミアムな100%ウールフラットウーブンプレイドファブリック。</t>
+        </is>
+      </c>
       <c r="G13" s="1" t="inlineStr">
         <is>
           <t>Vintage Porsche Blue Plaid Fabric - 100% Wool Flatwoven Twill</t>
         </is>
       </c>
-      <c r="H13" s="1" t="n"/>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t>ヴィンテージ ポルシェ ブループレイド生地 - 100%ウール フラットウーブンツイル</t>
+        </is>
+      </c>
       <c r="I13" s="1" t="inlineStr">
         <is>
           <t>Discover premium 100% wool automotive fabric featuring the classic 1970s Porsche RSR blue tartan pattern. Durable, period-correct woven cloth for luxury interiors.</t>
         </is>
       </c>
-      <c r="J13" s="1" t="n"/>
+      <c r="J13" s="1" t="inlineStr">
+        <is>
+          <t>クラシックな1970年代ポルシェRSRブルータータンパターンを特徴とするプレミアム100%ウール自動車用生地。高級内装向けの耐久性のある時代考証織物。</t>
+        </is>
+      </c>
       <c r="K13" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8525.jpg</t>
@@ -1093,25 +1286,41 @@
           <t>PORSCHE VELOURS PINSTRIPE</t>
         </is>
       </c>
-      <c r="D14" s="1" t="n"/>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>ポルシェ ベロア ピンストライプ</t>
+        </is>
+      </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
           <t>It is a velvet-like fabric featuring a dense, cut-pile surface. This gives it an incredibly plush, soft-touch texture that was highly favored for luxury and executive sports car cabins in the 1980s</t>
         </is>
       </c>
-      <c r="F14" s="1" t="n"/>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>高密度なカットパイル表面を持つベルベットのような生地。1980年代の高級車およびエグゼクティブスポーツカーキャビンで高く評価された、非常に豪華でソフトなタッチのテクスチャー。</t>
+        </is>
+      </c>
       <c r="G14" s="1" t="inlineStr">
         <is>
           <t>Porsche 911 928 944 Pinstripe Velour Seat Cloth</t>
         </is>
       </c>
-      <c r="H14" s="1" t="n"/>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t>ポルシェ911 928 944 ピンストライプ ベロア シートクロス</t>
+        </is>
+      </c>
       <c r="I14" s="1" t="inlineStr">
         <is>
           <t>Vintage-style vertical pinstripe velour fabric for classic Porsche interiors. Perfect for high-end seat insert and door card restorations.</t>
         </is>
       </c>
-      <c r="J14" s="1" t="n"/>
+      <c r="J14" s="1" t="inlineStr">
+        <is>
+          <t>クラシックポルシェ内装向けヴィンテージスタイルの縦ピンストライプベロア生地。高級シートインサートおよびドアカードレストアに最適。</t>
+        </is>
+      </c>
       <c r="K14" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA3217.jpg</t>
@@ -1138,25 +1347,41 @@
           <t>PORSCHE STUDIO</t>
         </is>
       </c>
-      <c r="D15" s="1" t="n"/>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>ポルシェ スタジオ</t>
+        </is>
+      </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
           <t>This is an authentic reproduction of Porsche’s iconic "Studio Check" automotive upholstery fabric, specifically curated for  Porsche 911 Carrera (964/993 generations), Porsche 928, and Porsche 968</t>
         </is>
       </c>
-      <c r="F15" s="1" t="n"/>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>ポルシェ911カレラ（964/993世代）、ポルシェ928、ポルシェ968向けにキュレーションされた、ポルシェの象徴的な「スタジオチェック」自動車用張り地の本格的な復刻版。</t>
+        </is>
+      </c>
       <c r="G15" s="1" t="inlineStr">
         <is>
           <t>Porsche Studio Check Grey Fabric | 964 993 928 Restoration Cloth</t>
         </is>
       </c>
-      <c r="H15" s="1" t="n"/>
+      <c r="H15" s="1" t="inlineStr">
+        <is>
+          <t>ポルシェ スタジオチェック グレー生地 | 964 993 928 レストアクロス</t>
+        </is>
+      </c>
       <c r="I15" s="1" t="inlineStr">
         <is>
           <t>Vintage Authentic reproduction of the classic Porsche Studio Check upholstery fabric</t>
         </is>
       </c>
-      <c r="J15" s="1" t="n"/>
+      <c r="J15" s="1" t="inlineStr">
+        <is>
+          <t>クラシックポルシェスタジオチェック張り地のヴィンテージ本格復刻版。</t>
+        </is>
+      </c>
       <c r="K15" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8118.jpg</t>
@@ -1183,25 +1408,41 @@
           <t>PORSCHE TARTAN</t>
         </is>
       </c>
-      <c r="D16" s="1" t="n"/>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>ポルシェ タータン</t>
+        </is>
+      </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Introduced in 1975, this legendary pattern was famously optioned on the early Porsche 911 Turbo (930) and the 911SC</t>
         </is>
       </c>
-      <c r="F16" s="1" t="n"/>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>1975年に導入されたこの伝説的なパターンは、アーリーポルシェ911ターボ（930）と911SCに有名なオプションとして採用されました。</t>
+        </is>
+      </c>
       <c r="G16" s="1" t="inlineStr">
         <is>
           <t>Porsche Classic Tartan Fabric | 911SC &amp; 930 Turbo Seat Cloth</t>
         </is>
       </c>
-      <c r="H16" s="1" t="n"/>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t>ポルシェ クラシック タータン生地 | 911SC &amp; 930ターボ シートクロス</t>
+        </is>
+      </c>
       <c r="I16" s="1" t="inlineStr">
         <is>
           <t>Vintage-style  plaid upholstery cloth for classic Porsche interiors. Durable, period-correct flatwoven check fabric for seats and door cards.</t>
         </is>
       </c>
-      <c r="J16" s="1" t="n"/>
+      <c r="J16" s="1" t="inlineStr">
+        <is>
+          <t>クラシックポルシェ内装向けヴィンテージスタイルのプレイド張り地クロス。シートおよびドアカード用の耐久性のある時代考証フラットウーブンチェック生地。</t>
+        </is>
+      </c>
       <c r="K16" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8217.jpg</t>
@@ -1228,25 +1469,41 @@
           <t>SELETED PLAID</t>
         </is>
       </c>
-      <c r="D17" s="1" t="n"/>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>セレクテッド プレイド</t>
+        </is>
+      </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
           <t>Selected plaid for automotive seat upholstery</t>
         </is>
       </c>
-      <c r="F17" s="1" t="n"/>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>自動車シート張り地向けセレクトプレイド。</t>
+        </is>
+      </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Automotive Plaid for Seat Upholstery </t>
         </is>
       </c>
-      <c r="H17" s="1" t="n"/>
+      <c r="H17" s="1" t="inlineStr">
+        <is>
+          <t>自動車用プレイド シート張り地</t>
+        </is>
+      </c>
       <c r="I17" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Polyester automtive plaid for seat upholstery </t>
         </is>
       </c>
-      <c r="J17" s="1" t="n"/>
+      <c r="J17" s="1" t="inlineStr">
+        <is>
+          <t>自動車シート張り地向けポリエステルプレイド。</t>
+        </is>
+      </c>
       <c r="K17" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA8517.jpg</t>
@@ -1273,25 +1530,41 @@
           <t>SPIRIT OF LE MANS</t>
         </is>
       </c>
-      <c r="D18" s="1" t="n"/>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>スピリット・オブ・ル・マン</t>
+        </is>
+      </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
           <t>The Spirit of Le Mans (SOLM) Wool Line is a premium, motorsport-inspired tartan collection woven in Scotland and engineered specifically for high-end automotive interiors. 100% premium wool woven in a durable 2/2 twill, featuring a heavy-duty weight of 500 glm (365 gsm). Pre-treated with specialized Soil Resist and Fire Retardant (FR) compliance coatings tailored for automotive safety standards.</t>
         </is>
       </c>
-      <c r="F18" s="1" t="n"/>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t>Sprit of Le Mans（SOLM）ウールラインは、スコットランドで織られ、高級自動車内装専用に設計された、モータースポーツにインスパイアされたプレミアムタータンコレクション。100%プレミアムウール、耐久性のある2/2ツイル織り、ヘビーデューティーウェイト500 glm（365 gsm）。自動車安全基準に適合した専用の防汚・難燃（FR）コーティング済み。</t>
+        </is>
+      </c>
       <c r="G18" s="1" t="inlineStr">
         <is>
           <t>100% Luxury Wool Automotive Fabric | Fire Retardant Tartan</t>
         </is>
       </c>
-      <c r="H18" s="1" t="n"/>
+      <c r="H18" s="1" t="inlineStr">
+        <is>
+          <t>100%高級ウール 自動車用生地 | 難燃タータン</t>
+        </is>
+      </c>
       <c r="I18" s="1" t="inlineStr">
         <is>
           <t>Heavyweight wool racing tartan cloth for luxury car interiors. Pre-treated with fire-retardant and soil-resist coatings. Woven in Scotland</t>
         </is>
       </c>
-      <c r="J18" s="1" t="n"/>
+      <c r="J18" s="1" t="inlineStr">
+        <is>
+          <t>高級車内装向けヘビーウェイトウールレーシングタータンクロス。難燃・防汚コーティング済み。スコットランド製。</t>
+        </is>
+      </c>
       <c r="K18" s="1" t="inlineStr">
         <is>
           <t>/uploads/fabric/Cover/FA2002.jpg</t>
@@ -1302,73 +1575,234 @@
       <c r="N18" s="1" t="n"/>
       <c r="O18" s="1" t="n"/>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="n"/>
-      <c r="B19" s="1" t="n"/>
-      <c r="C19" s="1" t="n"/>
+    <row r="19" ht="70" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>bmw-tartan</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>BMW TARTAN</t>
+        </is>
+      </c>
       <c r="D19" s="1" t="n"/>
-      <c r="E19" s="1" t="n"/>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>BMW ÜBERKARO is a classic tartan plaid fabric, famously known for its appearance in the legendary BMW E30 and the ultra-rare M3 Evolution II.</t>
+        </is>
+      </c>
       <c r="F19" s="1" t="n"/>
-      <c r="G19" s="1" t="n"/>
+      <c r="G19" s="1" t="inlineStr">
+        <is>
+          <t>Automotive Tartan Plaid Fabric, Upholstery for BMW E30 &amp; M3 Restoration</t>
+        </is>
+      </c>
       <c r="H19" s="1" t="n"/>
-      <c r="I19" s="1" t="n"/>
+      <c r="I19" s="1" t="inlineStr">
+        <is>
+          <t>Restore your classic BMW cabin with premium ÜBERKARO fabric. Woven to exact original specifications, this iconic E30 and M3 Evo II tartan plaid cloth matches the original factory pattern, color depth, and durability for a flawless showroom finish.</t>
+        </is>
+      </c>
       <c r="J19" s="1" t="n"/>
-      <c r="K19" s="1" t="n"/>
+      <c r="K19" s="1" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Cover/FA8275.jpeg</t>
+        </is>
+      </c>
       <c r="L19" s="1" t="n"/>
       <c r="M19" s="1" t="n"/>
       <c r="N19" s="1" t="n"/>
       <c r="O19" s="1" t="n"/>
     </row>
-    <row r="20">
-      <c r="A20" s="1" t="n"/>
-      <c r="B20" s="1" t="n"/>
-      <c r="C20" s="1" t="n"/>
+    <row r="20" ht="118" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>bmw-houndstooth</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>BMW HOUNDSTOOTH</t>
+        </is>
+      </c>
       <c r="D20" s="1" t="n"/>
-      <c r="E20" s="1" t="n"/>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>Restore classic BMW interiors with our premium German-reproduction Houndstooth (Pepita) seat cloth. This high-durability wool-blend fabric provides an authentic texture and finish for vintage BMW E10 (2002), E21, E28 (5 Series), and E30 (3 Series, including the 325i and early M3 variants). It is the ideal choice for concours-level seat center inserts, door cards, and complete interior restorations.</t>
+        </is>
+      </c>
       <c r="F20" s="1" t="n"/>
-      <c r="G20" s="1" t="n"/>
+      <c r="G20" s="1" t="inlineStr">
+        <is>
+          <t>BMW Houndstooth Fabric | Classic E30, E28, 2002 Upholstery Cloth</t>
+        </is>
+      </c>
       <c r="H20" s="1" t="n"/>
-      <c r="I20" s="1" t="n"/>
+      <c r="I20" s="1" t="inlineStr">
+        <is>
+          <t>Premium OEM-spec BMW Houndstooth (Pepita) seat fabric by the meter. Period-correct wool blend for classic E30, E28, and 2002 interior restoration.</t>
+        </is>
+      </c>
       <c r="J20" s="1" t="n"/>
-      <c r="K20" s="1" t="n"/>
+      <c r="K20" s="1" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Cover/FA1817.jpg</t>
+        </is>
+      </c>
       <c r="L20" s="1" t="n"/>
       <c r="M20" s="1" t="n"/>
       <c r="N20" s="1" t="n"/>
       <c r="O20" s="1" t="n"/>
     </row>
-    <row r="21">
-      <c r="A21" s="1" t="n"/>
-      <c r="B21" s="1" t="n"/>
-      <c r="C21" s="1" t="n"/>
+    <row r="21" ht="137" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>mercedes-houndstooth</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>MERCEDES HOUNDSTOOTH</t>
+        </is>
+      </c>
       <c r="D21" s="1" t="n"/>
-      <c r="E21" s="1" t="n"/>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>Restore the interior of your vintage W110 "Fintail" (Heckflosse) sedan with this premium reproduction houndstooth upholstery cloth. Woven to match the exact factory specifications of early 1960s mid-size Mercedes models, this dual-tone checkered fabric is a period-correct match for textile interiors in the 190c, 190Dc, and early 220 variants.</t>
+        </is>
+      </c>
       <c r="F21" s="1" t="n"/>
-      <c r="G21" s="1" t="n"/>
+      <c r="G21" s="1" t="inlineStr">
+        <is>
+          <t>Mercedes W110 Houndstooth Fabric | Vintage 190 &amp; 220 Seat Upholstery</t>
+        </is>
+      </c>
       <c r="H21" s="1" t="n"/>
-      <c r="I21" s="1" t="n"/>
+      <c r="I21" s="1" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz W110 Houndstooth seat cloth. Period-correct reproduction fabric for classic 190c, 190Dc, and 220 Fintail restoration by the meter.</t>
+        </is>
+      </c>
       <c r="J21" s="1" t="n"/>
-      <c r="K21" s="1" t="n"/>
+      <c r="K21" s="1" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Cover/FA8024.jpeg</t>
+        </is>
+      </c>
       <c r="L21" s="1" t="n"/>
       <c r="M21" s="1" t="n"/>
       <c r="N21" s="1" t="n"/>
       <c r="O21" s="1" t="n"/>
     </row>
-    <row r="22">
-      <c r="A22" s="1" t="n"/>
-      <c r="B22" s="1" t="n"/>
-      <c r="C22" s="1" t="n"/>
+    <row r="22" ht="168" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>vw-tartan</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>VW TARTAN</t>
+        </is>
+      </c>
       <c r="D22" s="1" t="n"/>
-      <c r="E22" s="1" t="n"/>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>Premium-reproduction Volkswagen T2 Westfalia upholstery fabric. Meticulously woven to match the exact factory specifications of the 1968–1979 Type 2 Campmobile models, this iconic checkered plaid utilizes a heavy-duty, dense weave</t>
+        </is>
+      </c>
       <c r="F22" s="1" t="n"/>
-      <c r="G22" s="1" t="n"/>
+      <c r="G22" s="1" t="inlineStr">
+        <is>
+          <t>VW T2 Westfalia Fabric | Classic Camper Plaid Seat Upholstery</t>
+        </is>
+      </c>
       <c r="H22" s="1" t="n"/>
-      <c r="I22" s="1" t="n"/>
+      <c r="I22" s="1" t="inlineStr">
+        <is>
+          <t>VW T2 Westfalia plaid camper upholstery fabric. Premium reproduction cloth for classic Bay Window rock-and-roll beds.</t>
+        </is>
+      </c>
       <c r="J22" s="1" t="n"/>
-      <c r="K22" s="1" t="n"/>
+      <c r="K22" s="1" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Cover/FA8715.jpeg</t>
+        </is>
+      </c>
       <c r="L22" s="1" t="n"/>
       <c r="M22" s="1" t="n"/>
       <c r="N22" s="1" t="n"/>
       <c r="O22" s="1" t="n"/>
+    </row>
+    <row r="23" ht="75" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>ferrari-technical</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>FERRARI TECHNICAL</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>フェラーリ テクニカル</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>Original Ferrari technical fabric used in 488 Pista, 812 Superfast etc. This synthetic textile prioritizes uncompromised motorsport performance over traditional luxury leather</t>
+        </is>
+      </c>
+      <c r="G23" s="1" t="inlineStr">
+        <is>
+          <t>Original Ferrari 488 Pista Technical Fabric | OEM Racing Seat Material</t>
+        </is>
+      </c>
+      <c r="I23" s="1" t="inlineStr">
+        <is>
+          <t>Source genuine Ferrari 488 Pista technical racing fabric. Perfect OEM-spec material for high-grip seat inserts, lightweight floor mats, and track upholstery.</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Cover/FA1269.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="K24" s="1" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Ferrari Technical/FA1269.jpeg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1381,7 +1815,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H86"/>
+  <dimension ref="A1:H111"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="34.1640625" customWidth="1" min="1" max="1"/>
@@ -4407,6 +4841,881 @@
       <c r="H86" t="inlineStr">
         <is>
           <t>イギリス</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>bmw-tartan</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>1</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>1.0mm</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>1.0mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>bmw-tartan</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>2</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>bmw-tartan</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>3</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>bmw-tartan</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>4</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Wool/Polyester</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>ウール/ポリエステル</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>bmw-tartan</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>5</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="15" customHeight="1">
+      <c r="A92" s="1" t="inlineStr">
+        <is>
+          <t>bmw-houndstooth</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>1</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>1.1mm</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>1.1mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="15" customHeight="1">
+      <c r="A93" s="1" t="inlineStr">
+        <is>
+          <t>bmw-houndstooth</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>2</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="15" customHeight="1">
+      <c r="A94" s="1" t="inlineStr">
+        <is>
+          <t>bmw-houndstooth</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>3</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="15" customHeight="1">
+      <c r="A95" s="1" t="inlineStr">
+        <is>
+          <t>bmw-houndstooth</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>4</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Wool/Polyester</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>ウール/ポリエステル</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="15" customHeight="1">
+      <c r="A96" s="1" t="inlineStr">
+        <is>
+          <t>bmw-houndstooth</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>5</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="15" customHeight="1">
+      <c r="A97" s="1" t="inlineStr">
+        <is>
+          <t>mercedes-houndstooth</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>1</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>1.0mm</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>1.0mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="15" customHeight="1">
+      <c r="A98" s="1" t="inlineStr">
+        <is>
+          <t>mercedes-houndstooth</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>2</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="15" customHeight="1">
+      <c r="A99" s="1" t="inlineStr">
+        <is>
+          <t>mercedes-houndstooth</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>3</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="15" customHeight="1">
+      <c r="A100" s="1" t="inlineStr">
+        <is>
+          <t>mercedes-houndstooth</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>4</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Wool</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>ウール</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="15" customHeight="1">
+      <c r="A101" s="1" t="inlineStr">
+        <is>
+          <t>mercedes-houndstooth</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>5</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="15" customHeight="1">
+      <c r="A102" s="1" t="inlineStr">
+        <is>
+          <t>vw-tartan</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>1</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>0.9mm</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>0.9mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="15" customHeight="1">
+      <c r="A103" s="1" t="inlineStr">
+        <is>
+          <t>vw-tartan</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>2</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="15" customHeight="1">
+      <c r="A104" s="1" t="inlineStr">
+        <is>
+          <t>vw-tartan</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>3</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="15" customHeight="1">
+      <c r="A105" s="1" t="inlineStr">
+        <is>
+          <t>vw-tartan</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>4</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Polyester</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>ポリエステル</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="15" customHeight="1">
+      <c r="A106" s="1" t="inlineStr">
+        <is>
+          <t>vw-tartan</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>5</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="15" customHeight="1">
+      <c r="A107" s="1" t="inlineStr">
+        <is>
+          <t>ferrari-technical</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>1</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>thickness</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>THICKNESS</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>厚さ</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>0.85mm</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>0.9mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="15" customHeight="1">
+      <c r="A108" s="1" t="inlineStr">
+        <is>
+          <t>ferrari-technical</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>2</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>自動車用</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="15" customHeight="1">
+      <c r="A109" s="1" t="inlineStr">
+        <is>
+          <t>ferrari-technical</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>3</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>WIDTH</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>140cm</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>140CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="15" customHeight="1">
+      <c r="A110" s="1" t="inlineStr">
+        <is>
+          <t>ferrari-technical</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>4</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>素材</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Polyester</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>ポリエステル</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="15" customHeight="1">
+      <c r="A111" s="1" t="inlineStr">
+        <is>
+          <t>ferrari-technical</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>5</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>country of origin</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>COUNTRY OF ORIGIN</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>製造国</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>ドイツ</t>
         </is>
       </c>
     </row>
@@ -4503,12 +5812,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q41"/>
+  <dimension ref="A1:Q55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="20.1640625" customWidth="1" min="3" max="3"/>
     <col width="36.83203125" customWidth="1" min="5" max="5"/>
     <col width="21.33203125" customWidth="1" min="6" max="6"/>
+    <col width="65.83203125" customWidth="1" min="8" max="8"/>
+    <col width="58.5" customWidth="1" min="9" max="9"/>
     <col width="35.83203125" customWidth="1" min="10" max="10"/>
     <col width="25" customWidth="1" min="11" max="11"/>
     <col width="30.1640625" customWidth="1" min="12" max="13"/>
@@ -6249,7 +7560,7 @@
         </is>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="240" customHeight="1">
       <c r="A37" t="inlineStr">
         <is>
           <t>fa8517</t>
@@ -6290,13 +7601,28 @@
           <t>/uploads/fabric/Preview/FA8517.jpg</t>
         </is>
       </c>
+      <c r="K37" s="1" t="inlineStr">
+        <is>
+          <t>Bespoke automotive seats with this premium foamed fabric. It is inspired directly by the historic legacy of the Porsche Sonderwunsch . Showcased as the defining pattern of the 992-generation 911 Turbo Sonderwunsch edition, this textile reimagines the iconic 1974 "Louise" Turbo No. 1 heritage cabin layout with a striking red, blue, and black checkered weave.</t>
+        </is>
+      </c>
+      <c r="M37" s="1" t="inlineStr">
+        <is>
+          <t>Porsche Sonderwunsch Fabric | Red Blue Black Plaid Upholstery</t>
+        </is>
+      </c>
+      <c r="O37" s="1" t="inlineStr">
+        <is>
+          <t>Premium OEM-spec Porsche Sonderwunsch program red, blue, and black plaid fabric. Foam-backed heritage seat cloth for custom 911 interior</t>
+        </is>
+      </c>
       <c r="Q37" t="inlineStr">
         <is>
           <t>/uploads/fabric/Selected Plaid/FA8517.jpg</t>
         </is>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="120" customHeight="1">
       <c r="A38" t="inlineStr">
         <is>
           <t>fa8553</t>
@@ -6337,16 +7663,31 @@
           <t>/uploads/fabric/Preview/FA8553.jpg</t>
         </is>
       </c>
+      <c r="K38" s="1" t="inlineStr">
+        <is>
+          <t>Premium reproduction "Carla" check upholstery fabric, famously featured in the late 1970s and 1980s Ford Capri S models (Mk2 and Mk3)</t>
+        </is>
+      </c>
+      <c r="M38" s="1" t="inlineStr">
+        <is>
+          <t>Ford Capri S Carla Fabric | Classic Orange &amp; Grey Plaid Upholstery</t>
+        </is>
+      </c>
+      <c r="O38" s="1" t="inlineStr">
+        <is>
+          <t>Ford Capri S "Carla" check seat fabric. Premium orange, grey, and black reproduction cloth for classic Mk2 &amp; Mk3 Capri interior restoration</t>
+        </is>
+      </c>
       <c r="Q38" t="inlineStr">
         <is>
           <t>/uploads/fabric/Selected Plaid/FA8553.jpg</t>
         </is>
       </c>
     </row>
-    <row r="39">
+    <row r="39" ht="210" customHeight="1">
       <c r="A39" t="inlineStr">
         <is>
-          <t>fa2002</t>
+          <t>fa8075</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6356,44 +7697,59 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>spirit-of-le-mans</t>
+          <t>selected-plaid</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>FA2002</t>
+          <t>FA8075</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>BLUE/NAVY/RED</t>
+          <t>GRAY/BLUE</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Spirit of Le Mans/FA2002.jpg</t>
+          <t>/uploads/fabric/Selected Plaid/FA8075.jpg</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Spirit of Le Mans/FA2002.jpg</t>
+          <t>/uploads/fabric/Selected Plaid/FA8075.jpg</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Preview/FA2002.jpg</t>
+          <t>/uploads/fabric/Preview/FA8075.jpeg</t>
+        </is>
+      </c>
+      <c r="K39" s="1" t="inlineStr">
+        <is>
+          <t>Restore the authentic interior of late-production Mexican-built Volkswagen Beetles—variously known as the Käfer, Kever, or Coccinelle—with our premium reproduction upholstery fabric which replicates the exact factory texture of the late 1970s through the 1980s Puebla production era</t>
+        </is>
+      </c>
+      <c r="M39" s="1" t="inlineStr">
+        <is>
+          <t>VW Beetle Mexico Heavy-duty Fabric | Classic Käfer &amp; Coccinelle Upholstery</t>
+        </is>
+      </c>
+      <c r="O39" s="1" t="inlineStr">
+        <is>
+          <t>VW Beetle Mexico (Käfer/Kever) striped heavy-duty seat fabric . Premium reproduction cloth for classic Puebla-built interiors.</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Spirit of Le Mans/FA2002.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
+          <t>/uploads/fabric/Selected Plaid/FA8075.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="105" customHeight="1">
       <c r="A40" t="inlineStr">
         <is>
-          <t>fa2202</t>
+          <t>fa8072</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -6403,84 +7759,817 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>spirit-of-le-mans</t>
+          <t>selected-plaid</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>FA2202</t>
+          <t>FA8072</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>BLUE/ORANGE/NAVY</t>
+          <t>BLACK/WHITE</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Spirit of Le Mans/FA2202.jpg</t>
+          <t>/uploads/fabric/Selected Plaid/FA8072.jpg</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Spirit of Le Mans/FA2202.jpg</t>
+          <t>/uploads/fabric/Selected Plaid/FA8072.jpg</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Preview/FA2202.jpg</t>
+          <t>/uploads/fabric/Preview/FA8072.jpeg</t>
+        </is>
+      </c>
+      <c r="K40" s="1" t="inlineStr">
+        <is>
+          <t>upgrade your modern classic with our premium Satellite Grey upholstery material, engineered specifically for the third-generation MINI Cooper  (F56)</t>
+        </is>
+      </c>
+      <c r="M40" s="1" t="inlineStr">
+        <is>
+          <t>MINI F56 Satellite Grey Fabric | MINI Cooper Seat Upholstery Material</t>
+        </is>
+      </c>
+      <c r="O40" s="1" t="inlineStr">
+        <is>
+          <t>Premium OEM-spec MINI F56 Satellite Grey cloth. Perfect for third-gen Cooper &amp; Cooper S seat and door panel restorations.</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>/uploads/fabric/Spirit of Le Mans/FA2202.jpg</t>
+          <t>/uploads/fabric/Selected Plaid/FA8072.jpg</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>fa2002</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>spirit-of-le-mans</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>FA2002</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>BLUE/NAVY/RED</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2002.jpg</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2002.jpg</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA2002.jpg</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2002.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>fa2202</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>spirit-of-le-mans</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>FA2202</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>BLUE/ORANGE/NAVY</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2202.jpg</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2202.jpg</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA2202.jpg</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Spirit of Le Mans/FA2202.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>fa2729</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>spirit-of-le-mans</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>FA2729</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>BLUE/BLACK/RED</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>/uploads/fabric/Spirit of Le Mans/FA2729.jpg</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>/uploads/fabric/Spirit of Le Mans/FA2729.jpg</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="J43" t="inlineStr">
         <is>
           <t>/uploads/fabric/Preview/FA2729.jpg</t>
         </is>
       </c>
-      <c r="Q41" t="inlineStr">
+      <c r="Q43" t="inlineStr">
         <is>
           <t>/uploads/fabric/Spirit of Le Mans/FA2729.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="15" customHeight="1">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>fa1817</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>bmw-houndstooth</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>FA1817</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>DARK GRAY</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW Houndstooth/FA1817.jpg</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW Houndstooth/FA1817.jpg</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA1817.jpg</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW Houndstooth/FA1817.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="15" customHeight="1">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>fa1815</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>bmw-houndstooth</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>FA1815</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LIGHT GRAY</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW Houndstooth/FA1815.jpg</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW Houndstooth/FA1815.jpg</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA1815.jpg</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW Houndstooth/FA1815.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="15" customHeight="1">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>fa8275</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C46" s="1" t="inlineStr">
+        <is>
+          <t>bmw-tartan</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>FA8275</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>BROWN/WHITE</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW Tartan/FA8275.jpg</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW Tartan/FA8275.jpg</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8275.jpeg</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW Tartan/FA8275.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="15" customHeight="1">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>fa9368</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>bmw-tartan</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>FA9368</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>BLACK/WHITE</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW Tartan/FA9368.jpg</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW Tartan/FA9368.jpg</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA9368.jpeg</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/BMW Tartan/FA9368.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>fa8024</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C48" s="1" t="inlineStr">
+        <is>
+          <t>mercedes-houndstooth</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>FA8024</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>BLUE/WHITE</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Houndstooth/FA8024.jpg</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Houndstooth/FA8024.jpg</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8024.jpeg</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Houndstooth/FA8024.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>fa8066</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C49" s="1" t="inlineStr">
+        <is>
+          <t>mercedes-houndstooth</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>FA8066</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>BLACK/BEIGE</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Houndstooth/FA8066.jpg</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Houndstooth/FA8066.jpg</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8066.jpeg</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Mercedes Houndstooth/FA8066.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="15" customHeight="1">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>fa8715</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C50" s="1" t="inlineStr">
+        <is>
+          <t>vw-tartan</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>FA8715</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ORAGNE/YELLOW</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/VW Tartan/FA8715.jpg</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/VW Tartan/FA8715.jpg</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8715.jpeg</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/VW Tartan/FA8715.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="15" customHeight="1">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>fa8726</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C51" s="1" t="inlineStr">
+        <is>
+          <t>vw-tartan</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>FA8726</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>BLUE/GREEN</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/VW Tartan/FA8726.jpg</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/VW Tartan/FA8726.jpg</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8726.jpeg</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/VW Tartan/FA8726.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="15" customHeight="1">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>fa8734</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C52" s="1" t="inlineStr">
+        <is>
+          <t>vw-tartan</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>FA8734</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>GREEN/YELLOW</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/VW Tartan/FA8734.jpg</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/VW Tartan/FA8734.jpg</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8734.jpeg</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/VW Tartan/FA8734.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="15" customHeight="1">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>fa8754</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C53" s="1" t="inlineStr">
+        <is>
+          <t>vw-tartan</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>FA8754</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>BROWN/BEIGE</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/VW Tartan/FA8754.jpg</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/VW Tartan/FA8754.jpg</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA8754.jpeg</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/VW Tartan/FA8754.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="90" customHeight="1">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ferrari-technical-fa1228</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ferrari-technical</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>FA1228</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>FA1228</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>FA1228</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>#111111</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Ferrari Technical/FA1228.jpg</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Ferrari Technical/FA1228.jpg</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA1228.jpeg</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Ferrari technical fabric for performance-oriented automotive interiors.</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>パフォーマンス志向の自動車内装向けフェラーリ テクニカルファブリック。</t>
+        </is>
+      </c>
+      <c r="M54" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Ferrari Technical Blue Fabric FR | 488 Pista Racing Seat Insert and Floor Mat</t>
+        </is>
+      </c>
+      <c r="O54" s="1" t="inlineStr">
+        <is>
+          <t>Orignal Ferrari technical black fabric for racing seat inserts and automotive upholstery.</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Ferrari Technical/FA1228.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="75" customHeight="1">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>ferrari-technical-fa1269</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>fabric</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>ferrari-technical</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>FA1269</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>FA1269</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>FA1269</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>#1d1d1d</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Ferrari Technical/FA1269.jpg</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Ferrari Technical/FA1269.jpg</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Preview/FA1269.jpeg</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Ferrari technical fabric for performance-oriented automotive interiors.</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>パフォーマンス志向の自動車内装向けフェラーリ テクニカルファブリック。</t>
+        </is>
+      </c>
+      <c r="M55" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Ferrari Technical Black Fabric FR | 488 Pista Racing Seat Insert and Floor Mat</t>
+        </is>
+      </c>
+      <c r="O55" s="1" t="inlineStr">
+        <is>
+          <t>Orignal Ferrari technical fabric for racing seat inserts and automotive upholstery.</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Ferrari Technical/FA1269.jpg</t>
         </is>
       </c>
     </row>
@@ -6597,8 +8686,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <cols>
+    <col width="14.6640625" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -7224,6 +9316,471 @@
       <c r="C41" t="inlineStr">
         <is>
           <t>/uploads/fabric/Case/FA2729.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>fa2002</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>2</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA2002.JPG</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>fa2202</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA2202.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>fa2729</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA2729-2.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>fa2729</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>3</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA2729-3.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>fa2729</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>4</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA2729.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>fa3018</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA3018.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>fa3132</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA3132.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>fa5990</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/ FA5990.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>fa8045</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA8045.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>fa8063</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA8063.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>fa8065</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>2</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA8065.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>fa8074</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA8074-2.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>fa8074</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>3</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA8074.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>fa8093</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA8093.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>fa8118</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>2</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA8118.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>fa8165</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/ FA8165-2.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>fa8165</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>3</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/ FA8165.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>fa8271</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>2</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA8271-2.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>fa8271</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>3</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA8271-3.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>fa8271</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>4</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA8271.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>fa8354</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>2</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA8354-2.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>fa8354</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA8354.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>fa8475</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>2</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA8475.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>fa8517</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>2</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA8517.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>fa8525</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>2</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA8525.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>fa8626</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>2</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA8626-2.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>fa8626</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>3</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA8626.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>ferrari-technical-fa1269</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>1</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA1269.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>ferrari-technical-fa1228</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA1228.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>ferrari-technical-fa1269</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>2</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA1269-2.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>ferrari-technical-fa1269</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>3</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>/uploads/fabric/Casephoto/FA1269-3.jpeg</t>
         </is>
       </c>
     </row>

</xml_diff>